<commit_message>
Finalize FOR-instance workflows and SAT results
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Ra6eac001f0ff4a30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rab9d308d1ec54165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="R190d1f3512194434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Ra0ef8c4b72634380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Reef70b203b1b4d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="R25955815a1c2420f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54,54 +54,51 @@
     <x:t xml:space="preserve">Brief note</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">FOR-instance Site Breakdown</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Held-out test metrics by CULS, NIBIO, RMIT, SCION and TUWIEN.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Site</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">FOR-instance</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">SegmentAnyTree</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">trained model</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">held-out test</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">CULS</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Stronger SAT site result.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">NIBIO</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">High recall but low precision; many background-confusion false positives.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RMIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Weak domain-transfer case with low recall and missed trees.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">SCION</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">TUWIEN</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">TreeX</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">FOR-instance Site Breakdown</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Held-out test metrics by CULS, NIBIO, RMIT, SCION and TUWIEN.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Site</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CULS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Stronger SAT site result.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NIBIO</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">High recall but low precision; many background-confusion false positives.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">RMIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weak domain-transfer case with low recall and missed trees.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">SCION</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TUWIEN</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Completed benchmark site result.</x:t>
   </x:si>
   <x:si>
@@ -145,9 +142,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">This is the mean IoU for matched predicted/reference tree segments.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Accepted SAT model. Test F1 is 0.480. Main weakness is over-segmentation/background confusion, especially NIBIO, TUWIEN and RMIT.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TreeX split</x:t>
@@ -160,8 +154,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="0.000"/>
+    <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -239,7 +234,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -257,6 +252,20 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -461,15 +470,15 @@
   <x:cols>
     <x:col min="1" max="1" width="12.6640625" style="2" customWidth="1"/>
     <x:col min="2" max="2" width="15.33203125" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="18.6640625" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="14.83203125" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="34" style="2" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" style="2" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="5.6640625" style="2" customWidth="1"/>
     <x:col min="6" max="6" width="13.6640625" style="2" customWidth="1"/>
     <x:col min="7" max="7" width="9.33203125" style="2" customWidth="1"/>
     <x:col min="8" max="8" width="6.5" style="2" customWidth="1"/>
     <x:col min="9" max="9" width="14" style="2" customWidth="1"/>
     <x:col min="10" max="12" width="4.1640625" style="2" customWidth="1"/>
-    <x:col min="13" max="13" width="60.1640625" style="2" customWidth="1"/>
+    <x:col min="13" max="13" width="76" style="2" hidden="0" customWidth="1"/>
     <x:col min="14" max="16384" width="8.83203125" style="2" customWidth="0"/>
   </x:cols>
   <x:sheetData>
@@ -546,100 +555,169 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="16">
-      <x:c r="A6" s="5" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E6" s="6">
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="5" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="str">
+        <x:v>SegmentAnyTree</x:v>
+      </x:c>
+      <x:c r="C6" s="13" t="str">
+        <x:v>published pretrained (provisional)</x:v>
+      </x:c>
+      <x:c r="D6" s="13" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F6" s="7">
-        <x:v>0.4798180559855062</x:v>
-      </x:c>
-      <x:c r="G6" s="7">
-        <x:v>0.38177725766656873</x:v>
-      </x:c>
-      <x:c r="H6" s="7">
-        <x:v>0.68218318412397361</x:v>
-      </x:c>
-      <x:c r="I6" s="7">
-        <x:v>0.83902055760111349</x:v>
-      </x:c>
-      <x:c r="J6" s="6">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="K6" s="6">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="L6" s="6">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="M6" s="5"/>
-    </x:row>
-    <x:row r="7" ht="16">
-      <x:c r="A7" s="5" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="F6" s="9" t="n">
+        <x:v>0.21807908985391006</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="n">
+        <x:v>0.16305741426559733</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="n">
+        <x:v>0.3491194684944685</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="n">
+        <x:v>0.4360803197096021</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="n">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="L6" s="11" t="n">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="M6" s="13" t="str">
+        <x:v>Released checkpoint diagnostic; coordinate-rematched exports failed point-preservation audit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="5" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="str">
+        <x:v>SegmentAnyTree</x:v>
+      </x:c>
+      <x:c r="C7" s="13" t="str">
+        <x:v>trained from scratch</x:v>
+      </x:c>
+      <x:c r="D7" s="13" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="n">
+        <x:v>0.482488</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="n">
+        <x:v>0.380686</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="n">
+        <x:v>0.695416</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="n">
+        <x:v>0.839284</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="K7" s="11" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="L7" s="11" t="n">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="M7" s="13" t="str">
+        <x:v>Accepted aligned point-wise result; checkpoint sat_for_quicktune_to49_20260706_140730.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="5" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="str">
+        <x:v>SegmentAnyTree</x:v>
+      </x:c>
+      <x:c r="C8" s="13" t="str">
+        <x:v>fine-tuned follow-up (rejected)</x:v>
+      </x:c>
+      <x:c r="D8" s="13" t="str">
+        <x:v>held-out smoke subset</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F8" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="11" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="M8" s="13" t="str">
+        <x:v>Rejected follow-up; semantic trees present but aligned instance predictions were all background.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
         <x:v>unsupervised parameterised baseline</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E7" s="6">
+      <x:c r="D9" s="14" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F7" s="7">
-        <x:v>0.40217455383523271</x:v>
-      </x:c>
-      <x:c r="G7" s="7">
+      <x:c r="F9" s="10" t="n">
+        <x:v>0.4021745538352327</x:v>
+      </x:c>
+      <x:c r="G9" s="10" t="n">
         <x:v>0.33655672754365584</x:v>
       </x:c>
-      <x:c r="H7" s="7">
-        <x:v>0.63867715673636727</x:v>
-      </x:c>
-      <x:c r="I7" s="7">
-        <x:v>0.82906705957422022</x:v>
-      </x:c>
-      <x:c r="J7" s="6">
+      <x:c r="H9" s="10" t="n">
+        <x:v>0.6386771567363673</x:v>
+      </x:c>
+      <x:c r="I9" s="10" t="n">
+        <x:v>0.8290670595742202</x:v>
+      </x:c>
+      <x:c r="J9" s="12" t="n">
         <x:v>186</x:v>
       </x:c>
-      <x:c r="K7" s="6">
+      <x:c r="K9" s="12" t="n">
         <x:v>467</x:v>
       </x:c>
-      <x:c r="L7" s="6">
+      <x:c r="L9" s="12" t="n">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="M7" s="5" t="str">
+      <x:c r="M9" s="14" t="str">
         <x:v>Completed TreeX benchmark. Unsupervised parameterised baseline.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="5"/>
-      <x:c r="B8" s="5"/>
-      <x:c r="C8" s="5"/>
-      <x:c r="D8" s="5"/>
-      <x:c r="E8" s="6"/>
-      <x:c r="F8" s="7"/>
-      <x:c r="G8" s="7"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
-      <x:c r="J8" s="6"/>
-      <x:c r="K8" s="6"/>
-      <x:c r="L8" s="6"/>
-      <x:c r="M8" s="5"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -671,7 +749,7 @@
   <x:sheetData>
     <x:row r="1" ht="20">
       <x:c r="A1" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -688,7 +766,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -714,7 +792,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
         <x:v>5</x:v>
@@ -746,16 +824,16 @@
     </x:row>
     <x:row r="6" ht="16">
       <x:c r="A6" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6" s="6">
         <x:v>1</x:v>
@@ -782,21 +860,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="5" t="s">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E7" s="6">
         <x:v>6</x:v>
@@ -823,21 +901,21 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="M7" s="5" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E8" s="6">
         <x:v>1</x:v>
@@ -864,21 +942,21 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="M8" s="5" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E9" s="6">
         <x:v>2</x:v>
@@ -905,21 +983,21 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="M9" s="5" t="s">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E10" s="6">
         <x:v>1</x:v>
@@ -946,21 +1024,21 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="M10" s="5" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E11" s="6">
         <x:v>1</x:v>
@@ -987,21 +1065,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M11" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E12" s="6">
         <x:v>6</x:v>
@@ -1028,21 +1106,21 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="M12" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E13" s="6">
         <x:v>1</x:v>
@@ -1069,21 +1147,21 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="M13" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>28</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E14" s="6">
         <x:v>2</x:v>
@@ -1110,21 +1188,21 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="M14" s="5" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D15" s="5" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E15" s="6">
         <x:v>1</x:v>
@@ -1151,16 +1229,16 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="M15" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="16">
       <x:c r="A16" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B16" s="5"/>
       <x:c r="C16" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D16" s="5"/>
       <x:c r="E16" s="6"/>
@@ -1175,11 +1253,11 @@
     </x:row>
     <x:row r="17" ht="16">
       <x:c r="A17" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B17" s="5"/>
       <x:c r="C17" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D17" s="5"/>
       <x:c r="E17" s="6"/>
@@ -1194,11 +1272,11 @@
     </x:row>
     <x:row r="18" ht="16">
       <x:c r="A18" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="5"/>
       <x:c r="C18" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D18" s="5"/>
       <x:c r="E18" s="6"/>
@@ -1213,11 +1291,11 @@
     </x:row>
     <x:row r="19" ht="16">
       <x:c r="A19" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B19" s="5"/>
       <x:c r="C19" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D19" s="5"/>
       <x:c r="E19" s="6"/>
@@ -1232,11 +1310,11 @@
     </x:row>
     <x:row r="20" ht="16">
       <x:c r="A20" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B20" s="5"/>
       <x:c r="C20" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D20" s="5"/>
       <x:c r="E20" s="6"/>
@@ -1251,11 +1329,11 @@
     </x:row>
     <x:row r="21" ht="16">
       <x:c r="A21" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B21" s="5"/>
       <x:c r="C21" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D21" s="5"/>
       <x:c r="E21" s="6"/>
@@ -1270,11 +1348,11 @@
     </x:row>
     <x:row r="22" ht="16">
       <x:c r="A22" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B22" s="5"/>
       <x:c r="C22" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D22" s="5"/>
       <x:c r="E22" s="6"/>
@@ -1289,11 +1367,11 @@
     </x:row>
     <x:row r="23" ht="16">
       <x:c r="A23" s="5" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="5"/>
       <x:c r="C23" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D23" s="5"/>
       <x:c r="E23" s="6"/>
@@ -1332,7 +1410,7 @@
   <x:sheetData>
     <x:row r="1" ht="20">
       <x:c r="A1" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -1340,7 +1418,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1348,25 +1426,25 @@
     </x:row>
     <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="D5" s="8" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="s">
+      <x:c r="E5" s="8" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="E5" s="8" t="s">
+      <x:c r="F5" s="8" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="s">
+      <x:c r="G5" s="8" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="G5" s="8" t="s">
+      <x:c r="H5" s="8" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="H5" s="8" t="s">
-        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
@@ -1374,10 +1452,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6">
         <x:v>1</x:v>
@@ -1394,13 +1472,13 @@
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>43</x:v>
-      </x:c>
       <x:c r="D7" t="s">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E7">
         <x:v>11</x:v>
@@ -1420,10 +1498,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E8">
         <x:v>1</x:v>
@@ -1440,13 +1518,13 @@
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>45</x:v>
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="str">
+        <x:v>Accepted SAT trained-from-dev model. Test F1 is 0.4825. The released checkpoint remains provisional, and the fine-tuned follow-up is rejected because it produced zero accepted instance predictions.</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>28</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E9">
         <x:v>3</x:v>
@@ -1463,13 +1541,13 @@
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="5" t="s">
-        <x:v>18</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
         <x:v>TreeX is an unsupervised parameterised baseline. Strict test F1 is 0.402.</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>29</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E10">
         <x:v>0</x:v>
@@ -1488,7 +1566,7 @@
       <x:c r="A11" s="5"/>
       <x:c r="B11" s="5"/>
       <x:c r="D11" s="8" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E11" s="8">
         <x:v>16</x:v>
@@ -1534,7 +1612,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="D15" s="8" t="s">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E15" s="8" t="s">
         <x:v>5</x:v>
@@ -1545,7 +1623,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="D16" t="s">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E16">
         <x:v>21</x:v>
@@ -1556,7 +1634,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="D17" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E17">
         <x:v>11</x:v>
@@ -1567,7 +1645,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="D18" t="s">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E18">
         <x:v>32</x:v>

</xml_diff>

<commit_message>
Align benchmark results and SAT comparison workflow
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Ra0ef8c4b72634380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Reef70b203b1b4d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="R25955815a1c2420f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Rc397d71b7cf343df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R7665de3c17e24ae3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="Rde5c19592c7c41fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,82 +66,58 @@
     <x:t xml:space="preserve">FOR-instance</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">SegmentAnyTree</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">held-out test</x:t>
+    <x:t xml:space="preserve">Notes</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Brief interpretation and workbook conventions.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Topic</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Note</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Site/type</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Train</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Validation</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Held-out test</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Overall</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">All main results use the held-out test split from the FOR-instance protocol.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">CULS</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Stronger SAT site result.</x:t>
+    <x:t xml:space="preserve">F1 definition</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Use F1 at IoU &gt;= 0.5 for the main comparison. TreeX uses strict F1 so extra predicted instances are penalised in the same spirit as SAT.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">NIBIO</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">High recall but low precision; many background-confusion false positives.</x:t>
+    <x:t xml:space="preserve">This is the mean IoU for matched predicted/reference tree segments.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">RMIT</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Weak domain-transfer case with low recall and missed trees.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">SCION</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TUWIEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">TreeX</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Completed benchmark site result.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Low baseline site result.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Notes</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Brief interpretation and workbook conventions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Topic</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Note</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Site/type</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Train</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Validation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Held-out test</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Overall</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">All main results use the held-out test split from the FOR-instance protocol.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">F1 definition</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use F1 at IoU &gt;= 0.5 for the main comparison. TreeX uses strict F1 so extra predicted instances are penalised in the same spirit as SAT.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">This is the mean IoU for matched predicted/reference tree segments.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TreeX split</x:t>
@@ -468,18 +444,21 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.6640625" style="2" customWidth="1"/>
-    <x:col min="2" max="2" width="15.33203125" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="34" style="2" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="14" style="2" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" style="2" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" style="2" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" style="2" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="5.6640625" style="2" customWidth="1"/>
-    <x:col min="6" max="6" width="13.6640625" style="2" customWidth="1"/>
-    <x:col min="7" max="7" width="9.33203125" style="2" customWidth="1"/>
-    <x:col min="8" max="8" width="6.5" style="2" customWidth="1"/>
-    <x:col min="9" max="9" width="14" style="2" customWidth="1"/>
+    <x:col min="5" max="5" width="7" style="2" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" style="2" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" style="2" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" style="2" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" style="2" hidden="0" customWidth="1"/>
     <x:col min="10" max="12" width="4.1640625" style="2" customWidth="1"/>
-    <x:col min="13" max="13" width="76" style="2" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="72" style="2" hidden="0" customWidth="1"/>
     <x:col min="14" max="16384" width="8.83203125" style="2" customWidth="0"/>
+    <x:col min="10" max="10" width="8" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="20">
@@ -555,7 +534,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="42" customHeight="1">
+    <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="5" t="str">
         <x:v>FOR-instance</x:v>
       </x:c>
@@ -563,7 +542,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C6" s="13" t="str">
-        <x:v>published pretrained (provisional)</x:v>
+        <x:v>published pretrained (current target)</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:v>held-out test</x:v>
@@ -571,32 +550,18 @@
       <x:c r="E6" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="n">
-        <x:v>0.21807908985391006</x:v>
-      </x:c>
-      <x:c r="G6" s="9" t="n">
-        <x:v>0.16305741426559733</x:v>
-      </x:c>
-      <x:c r="H6" s="9" t="n">
-        <x:v>0.3491194684944685</x:v>
-      </x:c>
-      <x:c r="I6" s="9" t="n">
-        <x:v>0.4360803197096021</x:v>
-      </x:c>
-      <x:c r="J6" s="11" t="n">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="K6" s="11" t="n">
-        <x:v>678</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="n">
-        <x:v>212</x:v>
-      </x:c>
+      <x:c r="F6" s="9"/>
+      <x:c r="G6" s="9"/>
+      <x:c r="H6" s="9"/>
+      <x:c r="I6" s="9"/>
+      <x:c r="J6" s="11"/>
+      <x:c r="K6" s="11"/>
+      <x:c r="L6" s="11"/>
       <x:c r="M6" s="13" t="str">
-        <x:v>Released checkpoint diagnostic; coordinate-rematched exports failed point-preservation audit.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
+        <x:v>Pending aligned evaluation of released checkpoint; no weight updates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="5" t="str">
         <x:v>FOR-instance</x:v>
       </x:c>
@@ -604,7 +569,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>trained from scratch</x:v>
+        <x:v>fine-tuned on development (current target)</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
         <x:v>held-out test</x:v>
@@ -612,32 +577,18 @@
       <x:c r="E7" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F7" s="9" t="n">
-        <x:v>0.482488</x:v>
-      </x:c>
-      <x:c r="G7" s="9" t="n">
-        <x:v>0.380686</x:v>
-      </x:c>
-      <x:c r="H7" s="9" t="n">
-        <x:v>0.695416</x:v>
-      </x:c>
-      <x:c r="I7" s="9" t="n">
-        <x:v>0.839284</x:v>
-      </x:c>
-      <x:c r="J7" s="11" t="n">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="K7" s="11" t="n">
-        <x:v>336</x:v>
-      </x:c>
-      <x:c r="L7" s="11" t="n">
-        <x:v>121</x:v>
-      </x:c>
+      <x:c r="F7" s="9"/>
+      <x:c r="G7" s="9"/>
+      <x:c r="H7" s="9"/>
+      <x:c r="I7" s="9"/>
+      <x:c r="J7" s="11"/>
+      <x:c r="K7" s="11"/>
+      <x:c r="L7" s="11"/>
       <x:c r="M7" s="13" t="str">
-        <x:v>Accepted aligned point-wise result; checkpoint sat_for_quicktune_to49_20260706_140730.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="42" customHeight="1">
+        <x:v>Pending released-weight fine-tuning, development validation and aligned test evaluation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="5" t="str">
         <x:v>FOR-instance</x:v>
       </x:c>
@@ -645,48 +596,48 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C8" s="13" t="str">
-        <x:v>fine-tuned follow-up (rejected)</x:v>
+        <x:v>published pretrained (historical provisional)</x:v>
       </x:c>
       <x:c r="D8" s="13" t="str">
-        <x:v>held-out smoke subset</x:v>
+        <x:v>held-out test</x:v>
       </x:c>
       <x:c r="E8" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>0.21807908985391006</x:v>
       </x:c>
       <x:c r="G8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>0.16305741426559733</x:v>
       </x:c>
       <x:c r="H8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>0.3491194684944685</x:v>
       </x:c>
       <x:c r="I8" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>0.4360803197096021</x:v>
       </x:c>
       <x:c r="J8" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="K8" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="L8" s="11" t="n">
-        <x:v>50</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="M8" s="13" t="str">
-        <x:v>Rejected follow-up; semantic trees present but aligned instance predictions were all background.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="42" customHeight="1">
+        <x:v>Coordinate-rematched diagnostic retained; exports failed point-preservation audit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" t="str">
         <x:v>FOR-instance</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>TreeX</x:v>
+        <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>unsupervised parameterised baseline</x:v>
+        <x:v>trained from scratch (historical)</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
         <x:v>held-out test</x:v>
@@ -695,28 +646,110 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="F9" s="10" t="n">
-        <x:v>0.4021745538352327</x:v>
+        <x:v>0.4825</x:v>
       </x:c>
       <x:c r="G9" s="10" t="n">
-        <x:v>0.33655672754365584</x:v>
+        <x:v>0.3807</x:v>
       </x:c>
       <x:c r="H9" s="10" t="n">
-        <x:v>0.6386771567363673</x:v>
+        <x:v>0.6954</x:v>
       </x:c>
       <x:c r="I9" s="10" t="n">
-        <x:v>0.8290670595742202</x:v>
+        <x:v>0.839284</x:v>
       </x:c>
       <x:c r="J9" s="12" t="n">
-        <x:v>186</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="K9" s="12" t="n">
-        <x:v>467</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="L9" s="12" t="n">
-        <x:v>137</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="M9" s="14" t="str">
-        <x:v>Completed TreeX benchmark. Unsupervised parameterised baseline.</x:v>
+        <x:v>Completed historical aligned result; not a current target. Micro F1 0.4692.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>SegmentAnyTree</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>rejected fine-tune (historical)</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>held-out smoke subset</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="12" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Rejected 8 July diagnostic; retained, but not used as the replacement fine-tune.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>unchanged deterministic baseline</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="n">
+        <x:v>0.38310765715157086</x:v>
+      </x:c>
+      <x:c r="G11" s="10" t="n">
+        <x:v>0.27105666156202146</x:v>
+      </x:c>
+      <x:c r="H11" s="10" t="n">
+        <x:v>0.5479876160990712</x:v>
+      </x:c>
+      <x:c r="I11" s="10" t="n">
+        <x:v>0.8037642651576798</x:v>
+      </x:c>
+      <x:c r="J11" s="12" t="n">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="K11" s="12" t="n">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="L11" s="12" t="n">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Completed aligned point-wise baseline; mean plot F1 shown, micro F1 0.3627.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -826,420 +859,416 @@
       <x:c r="A6" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
+      <x:c r="B6" s="5" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="n">
+        <x:v>0.5479452054794521</x:v>
+      </x:c>
+      <x:c r="G6" s="7" t="n">
+        <x:v>0.37735849056603776</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="n">
+        <x:v>0.9476273064944747</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="E6" s="6">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F6" s="7">
-        <x:v>0.54794520547945214</x:v>
-      </x:c>
-      <x:c r="G6" s="7">
-        <x:v>0.37735849056603776</x:v>
-      </x:c>
-      <x:c r="H6" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I6" s="7">
-        <x:v>0.94762730649447469</x:v>
-      </x:c>
-      <x:c r="J6" s="6">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K6" s="6">
+      <x:c r="K6" s="6" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="L6" s="6">
+      <x:c r="L6" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M6" s="5" t="s">
-        <x:v>21</x:v>
+      <x:c r="M6" s="5" t="str">
+        <x:v>Historical site result; retained for traceability.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E7" s="6">
+      <x:c r="B7" s="5" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C7" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D7" s="5" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F7" s="7">
+      <x:c r="F7" s="7" t="n">
         <x:v>0.47905399926507836</x:v>
       </x:c>
-      <x:c r="G7" s="7">
+      <x:c r="G7" s="7" t="n">
         <x:v>0.36172209807653116</x:v>
       </x:c>
-      <x:c r="H7" s="7">
-        <x:v>0.72159013650241721</x:v>
-      </x:c>
-      <x:c r="I7" s="7">
+      <x:c r="H7" s="7" t="n">
+        <x:v>0.7215901365024172</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="n">
         <x:v>0.8395179520359185</x:v>
       </x:c>
-      <x:c r="J7" s="6">
+      <x:c r="J7" s="6" t="n">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="K7" s="6">
+      <x:c r="K7" s="6" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="L7" s="6">
+      <x:c r="L7" s="6" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="M7" s="5" t="s">
-        <x:v>23</x:v>
+      <x:c r="M7" s="5" t="str">
+        <x:v>Historical site result; high recall with many false positives.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E8" s="6">
+      <x:c r="B8" s="5" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F8" s="7">
+      <x:c r="F8" s="7" t="n">
         <x:v>0.34426229508196726</x:v>
       </x:c>
-      <x:c r="G8" s="7">
-        <x:v>0.36206896551724138</x:v>
-      </x:c>
-      <x:c r="H8" s="7">
+      <x:c r="G8" s="7" t="n">
+        <x:v>0.3620689655172414</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="n">
         <x:v>0.328125</x:v>
       </x:c>
-      <x:c r="I8" s="7">
-        <x:v>0.77826505556998948</x:v>
-      </x:c>
-      <x:c r="J8" s="6">
+      <x:c r="I8" s="7" t="n">
+        <x:v>0.7782650555699895</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="K8" s="6">
+      <x:c r="K8" s="6" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="L8" s="6">
+      <x:c r="L8" s="6" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="M8" s="5" t="s">
-        <x:v>25</x:v>
+      <x:c r="M8" s="5" t="str">
+        <x:v>Historical site result; weak transfer and low recall.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="E9" s="6">
+      <x:c r="B9" s="5" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F9" s="7">
-        <x:v>0.64305750350631141</x:v>
-      </x:c>
-      <x:c r="G9" s="7">
-        <x:v>0.53378378378378377</x:v>
-      </x:c>
-      <x:c r="H9" s="7">
-        <x:v>0.80888888888888888</x:v>
-      </x:c>
-      <x:c r="I9" s="7">
-        <x:v>0.91226977751388616</x:v>
-      </x:c>
-      <x:c r="J9" s="6">
+      <x:c r="F9" s="7" t="n">
+        <x:v>0.6430575035063114</x:v>
+      </x:c>
+      <x:c r="G9" s="7" t="n">
+        <x:v>0.5337837837837838</x:v>
+      </x:c>
+      <x:c r="H9" s="7" t="n">
+        <x:v>0.8088888888888889</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="n">
+        <x:v>0.9122697775138862</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="K9" s="6">
+      <x:c r="K9" s="6" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="L9" s="6">
+      <x:c r="L9" s="6" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="M9" s="5" t="s">
-        <x:v>21</x:v>
+      <x:c r="M9" s="5" t="str">
+        <x:v>Historical site result; strongest retained SAT site.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
+      <x:c r="B10" s="5" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="7" t="n">
+        <x:v>0.22535211267605634</x:v>
+      </x:c>
+      <x:c r="G10" s="7" t="n">
+        <x:v>0.2222222222222222</x:v>
+      </x:c>
+      <x:c r="H10" s="7" t="n">
+        <x:v>0.22857142857142856</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="n">
+        <x:v>0.6416865043044996</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="L10" s="6" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E10" s="6">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F10" s="7">
-        <x:v>0.22535211267605634</x:v>
-      </x:c>
-      <x:c r="G10" s="7">
-        <x:v>0.22222222222222221</x:v>
-      </x:c>
-      <x:c r="H10" s="7">
-        <x:v>0.22857142857142856</x:v>
-      </x:c>
-      <x:c r="I10" s="7">
-        <x:v>0.64168650430449958</x:v>
-      </x:c>
-      <x:c r="J10" s="6">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="K10" s="6">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="L10" s="6">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="M10" s="5" t="s">
-        <x:v>25</x:v>
+      <x:c r="M10" s="5" t="str">
+        <x:v>Historical site result; weak transfer and low recall.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="s">
+      <x:c r="B11" s="5" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F11" s="7" t="n">
+        <x:v>0.5797101449275363</x:v>
+      </x:c>
+      <x:c r="G11" s="7" t="n">
+        <x:v>0.40816326530612246</x:v>
+      </x:c>
+      <x:c r="H11" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="n">
+        <x:v>0.9384354128263748</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="E11" s="6">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F11" s="7">
-        <x:v>0.57971014492753625</x:v>
-      </x:c>
-      <x:c r="G11" s="7">
-        <x:v>0.4081632653061224</x:v>
-      </x:c>
-      <x:c r="H11" s="7">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I11" s="7">
-        <x:v>0.94048673335593758</x:v>
-      </x:c>
-      <x:c r="J11" s="6">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K11" s="6">
+      <x:c r="K11" s="6" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L11" s="6">
+      <x:c r="L11" s="6" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M11" s="5" t="s">
-        <x:v>29</x:v>
+      <x:c r="M11" s="5" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E12" s="6">
+      <x:c r="B12" s="5" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="F12" s="7">
-        <x:v>0.36511874809844286</x:v>
-      </x:c>
-      <x:c r="G12" s="7">
-        <x:v>0.24887458997316317</x:v>
-      </x:c>
-      <x:c r="H12" s="7">
-        <x:v>0.70041043549815463</x:v>
-      </x:c>
-      <x:c r="I12" s="7">
-        <x:v>0.8111017299666794</x:v>
-      </x:c>
-      <x:c r="J12" s="6">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="K12" s="6">
-        <x:v>346</x:v>
-      </x:c>
-      <x:c r="L12" s="6">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="M12" s="5" t="s">
-        <x:v>29</x:v>
+      <x:c r="F12" s="7" t="n">
+        <x:v>0.34632498065993217</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="n">
+        <x:v>0.23478260869565218</x:v>
+      </x:c>
+      <x:c r="H12" s="7" t="n">
+        <x:v>0.6708074534161491</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="n">
+        <x:v>0.7750563475089646</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="L12" s="6" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="M12" s="5" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E13" s="6">
+      <x:c r="B13" s="5" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C13" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D13" s="5" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F13" s="7">
-        <x:v>0.26506024096385539</x:v>
-      </x:c>
-      <x:c r="G13" s="7">
-        <x:v>0.57894736842105265</x:v>
-      </x:c>
-      <x:c r="H13" s="7">
-        <x:v>0.171875</x:v>
-      </x:c>
-      <x:c r="I13" s="7">
-        <x:v>0.8730110831608251</x:v>
-      </x:c>
-      <x:c r="J13" s="6">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="K13" s="6">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="L13" s="6">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="M13" s="5" t="s">
-        <x:v>30</x:v>
+      <x:c r="F13" s="7" t="n">
+        <x:v>0.216867469879518</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="n">
+        <x:v>0.47368421052631576</x:v>
+      </x:c>
+      <x:c r="H13" s="7" t="n">
+        <x:v>0.140625</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="n">
+        <x:v>0.8964955219132982</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="L13" s="6" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="M13" s="5" t="str">
+        <x:v>Low baseline site result.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
+      <x:c r="B14" s="5" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="n">
+        <x:v>0.5401987353206865</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="n">
+        <x:v>0.6046511627906976</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="n">
+        <x:v>0.8094268084447702</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="E14" s="6">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F14" s="7">
-        <x:v>0.56458897922312556</x:v>
-      </x:c>
-      <x:c r="G14" s="7">
-        <x:v>0.514992503748126</x:v>
-      </x:c>
-      <x:c r="H14" s="7">
-        <x:v>0.62555555555555564</x:v>
-      </x:c>
-      <x:c r="I14" s="7">
-        <x:v>0.83448179544437318</x:v>
-      </x:c>
-      <x:c r="J14" s="6">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="K14" s="6">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="L14" s="6">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="M14" s="5" t="s">
-        <x:v>29</x:v>
+      <x:c r="K14" s="6" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="L14" s="6" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="M14" s="5" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="5" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E15" s="6">
+      <x:c r="B15" s="5" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F15" s="7">
-        <x:v>0.25925925925925919</x:v>
-      </x:c>
-      <x:c r="G15" s="7">
-        <x:v>0.19178082191780821</x:v>
-      </x:c>
-      <x:c r="H15" s="7">
+      <x:c r="F15" s="7" t="n">
+        <x:v>0.2592592592592592</x:v>
+      </x:c>
+      <x:c r="G15" s="7" t="n">
+        <x:v>0.1917808219178082</x:v>
+      </x:c>
+      <x:c r="H15" s="7" t="n">
         <x:v>0.4</x:v>
       </x:c>
-      <x:c r="I15" s="7">
-        <x:v>0.77066586811083759</x:v>
-      </x:c>
-      <x:c r="J15" s="6">
+      <x:c r="I15" s="7" t="n">
+        <x:v>0.7372842800514755</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="K15" s="6">
+      <x:c r="K15" s="6" t="n">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="L15" s="6">
+      <x:c r="L15" s="6" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="M15" s="5" t="s">
-        <x:v>30</x:v>
+      <x:c r="M15" s="5" t="str">
+        <x:v>Low baseline site result.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="16">
-      <x:c r="A16" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A16" s="5"/>
       <x:c r="B16" s="5"/>
-      <x:c r="C16" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C16" s="5"/>
       <x:c r="D16" s="5"/>
       <x:c r="E16" s="6"/>
       <x:c r="F16" s="7"/>
@@ -1252,13 +1281,9 @@
       <x:c r="M16" s="5"/>
     </x:row>
     <x:row r="17" ht="16">
-      <x:c r="A17" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A17" s="5"/>
       <x:c r="B17" s="5"/>
-      <x:c r="C17" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C17" s="5"/>
       <x:c r="D17" s="5"/>
       <x:c r="E17" s="6"/>
       <x:c r="F17" s="7"/>
@@ -1271,13 +1296,9 @@
       <x:c r="M17" s="5"/>
     </x:row>
     <x:row r="18" ht="16">
-      <x:c r="A18" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A18" s="5"/>
       <x:c r="B18" s="5"/>
-      <x:c r="C18" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C18" s="5"/>
       <x:c r="D18" s="5"/>
       <x:c r="E18" s="6"/>
       <x:c r="F18" s="7"/>
@@ -1290,13 +1311,9 @@
       <x:c r="M18" s="5"/>
     </x:row>
     <x:row r="19" ht="16">
-      <x:c r="A19" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A19" s="5"/>
       <x:c r="B19" s="5"/>
-      <x:c r="C19" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C19" s="5"/>
       <x:c r="D19" s="5"/>
       <x:c r="E19" s="6"/>
       <x:c r="F19" s="7"/>
@@ -1309,13 +1326,9 @@
       <x:c r="M19" s="5"/>
     </x:row>
     <x:row r="20" ht="16">
-      <x:c r="A20" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A20" s="5"/>
       <x:c r="B20" s="5"/>
-      <x:c r="C20" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C20" s="5"/>
       <x:c r="D20" s="5"/>
       <x:c r="E20" s="6"/>
       <x:c r="F20" s="7"/>
@@ -1328,13 +1341,9 @@
       <x:c r="M20" s="5"/>
     </x:row>
     <x:row r="21" ht="16">
-      <x:c r="A21" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A21" s="5"/>
       <x:c r="B21" s="5"/>
-      <x:c r="C21" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C21" s="5"/>
       <x:c r="D21" s="5"/>
       <x:c r="E21" s="6"/>
       <x:c r="F21" s="7"/>
@@ -1347,13 +1356,9 @@
       <x:c r="M21" s="5"/>
     </x:row>
     <x:row r="22" ht="16">
-      <x:c r="A22" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A22" s="5"/>
       <x:c r="B22" s="5"/>
-      <x:c r="C22" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C22" s="5"/>
       <x:c r="D22" s="5"/>
       <x:c r="E22" s="6"/>
       <x:c r="F22" s="7"/>
@@ -1366,13 +1371,9 @@
       <x:c r="M22" s="5"/>
     </x:row>
     <x:row r="23" ht="16">
-      <x:c r="A23" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
+      <x:c r="A23" s="5"/>
       <x:c r="B23" s="5"/>
-      <x:c r="C23" s="5" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="C23" s="5"/>
       <x:c r="D23" s="5"/>
       <x:c r="E23" s="6"/>
       <x:c r="F23" s="7"/>
@@ -1410,7 +1411,7 @@
   <x:sheetData>
     <x:row r="1" ht="20">
       <x:c r="A1" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -1418,7 +1419,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>32</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1426,25 +1427,25 @@
     </x:row>
     <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
-        <x:v>33</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B5" s="4" t="s">
-        <x:v>34</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="8" t="s">
-        <x:v>35</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E5" s="8" t="s">
-        <x:v>36</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F5" s="8" t="s">
-        <x:v>37</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G5" s="8" t="s">
-        <x:v>38</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H5" s="8" t="s">
-        <x:v>39</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
@@ -1452,10 +1453,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>40</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E6">
         <x:v>1</x:v>
@@ -1472,13 +1473,13 @@
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
-        <x:v>41</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>42</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D7" t="s">
-        <x:v>22</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E7">
         <x:v>11</x:v>
@@ -1498,10 +1499,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>43</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>24</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E8">
         <x:v>1</x:v>
@@ -1517,14 +1518,14 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="16">
-      <x:c r="A9" s="5" t="s">
-        <x:v>18</x:v>
+      <x:c r="A9" s="5" t="str">
+        <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>Accepted SAT trained-from-dev model. Test F1 is 0.4825. The released checkpoint remains provisional, and the fine-tuned follow-up is rejected because it produced zero accepted instance predictions.</x:v>
+        <x:v>Current target: aligned released-checkpoint test, then released-weight fine-tuning on development data and aligned test. The completed from-scratch result (mean plot F1 0.4825; micro F1 0.4692) remains historical.</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>26</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E9">
         <x:v>3</x:v>
@@ -1540,14 +1541,14 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="16">
-      <x:c r="A10" s="5" t="s">
-        <x:v>28</x:v>
+      <x:c r="A10" s="5" t="str">
+        <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>TreeX is an unsupervised parameterised baseline. Strict test F1 is 0.402.</x:v>
+        <x:v>TreeX remains the completed deterministic baseline. Corrected union-mask test mean plot F1 is 0.3831 and micro F1 is 0.3627.</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>27</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E10">
         <x:v>0</x:v>
@@ -1566,7 +1567,7 @@
       <x:c r="A11" s="5"/>
       <x:c r="B11" s="5"/>
       <x:c r="D11" s="8" t="s">
-        <x:v>39</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E11" s="8">
         <x:v>16</x:v>
@@ -1612,7 +1613,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="D15" s="8" t="s">
-        <x:v>44</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E15" s="8" t="s">
         <x:v>5</x:v>
@@ -1623,7 +1624,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="D16" t="s">
-        <x:v>45</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E16">
         <x:v>21</x:v>
@@ -1634,7 +1635,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="D17" t="s">
-        <x:v>38</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E17">
         <x:v>11</x:v>
@@ -1645,7 +1646,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="D18" t="s">
-        <x:v>39</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E18">
         <x:v>32</x:v>

</xml_diff>

<commit_message>
Finalize SegmentAnyTree benchmark results
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Rc397d71b7cf343df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R7665de3c17e24ae3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="Rde5c19592c7c41fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R230dab76ef3e4539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Ra66e0dfcd851485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="R03da0b1830544b38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,9 +55,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">FOR-instance Site Breakdown</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Held-out test metrics by CULS, NIBIO, RMIT, SCION and TUWIEN.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Site</x:t>
@@ -542,7 +539,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C6" s="13" t="str">
-        <x:v>published pretrained (current target)</x:v>
+        <x:v>published pretrained (completed baseline)</x:v>
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:v>held-out test</x:v>
@@ -550,15 +547,29 @@
       <x:c r="E6" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F6" s="9"/>
-      <x:c r="G6" s="9"/>
-      <x:c r="H6" s="9"/>
-      <x:c r="I6" s="9"/>
-      <x:c r="J6" s="11"/>
-      <x:c r="K6" s="11"/>
-      <x:c r="L6" s="11"/>
+      <x:c r="F6" s="9" t="n">
+        <x:v>0.45340897930934665</x:v>
+      </x:c>
+      <x:c r="G6" s="9" t="n">
+        <x:v>0.32301693464050424</x:v>
+      </x:c>
+      <x:c r="H6" s="9" t="n">
+        <x:v>0.8085742004820952</x:v>
+      </x:c>
+      <x:c r="I6" s="9" t="n">
+        <x:v>0.8603003216196654</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="n">
+        <x:v>247</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="n">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="L6" s="11" t="n">
+        <x:v>76</x:v>
+      </x:c>
       <x:c r="M6" s="13" t="str">
-        <x:v>Pending aligned evaluation of released checkpoint; no weight updates.</x:v>
+        <x:v>Completed aligned baseline; micro F1 0.4442. Released training manifest remains unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -569,7 +580,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C7" s="13" t="str">
-        <x:v>fine-tuned on development (current target)</x:v>
+        <x:v>fine-tuned on development (primary)</x:v>
       </x:c>
       <x:c r="D7" s="13" t="str">
         <x:v>held-out test</x:v>
@@ -577,15 +588,29 @@
       <x:c r="E7" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F7" s="9"/>
-      <x:c r="G7" s="9"/>
-      <x:c r="H7" s="9"/>
-      <x:c r="I7" s="9"/>
-      <x:c r="J7" s="11"/>
-      <x:c r="K7" s="11"/>
-      <x:c r="L7" s="11"/>
+      <x:c r="F7" s="9" t="n">
+        <x:v>0.5446789009405125</x:v>
+      </x:c>
+      <x:c r="G7" s="9" t="n">
+        <x:v>0.4296635853788897</x:v>
+      </x:c>
+      <x:c r="H7" s="9" t="n">
+        <x:v>0.780590486248381</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="n">
+        <x:v>0.85847139408441</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="n">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="K7" s="11" t="n">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="L7" s="11" t="n">
+        <x:v>86</x:v>
+      </x:c>
       <x:c r="M7" s="13" t="str">
-        <x:v>Pending released-weight fine-tuning, development validation and aligned test evaluation.</x:v>
+        <x:v>Completed primary aligned result; micro F1 0.5320. Frozen one-time test evaluation.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -637,7 +662,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="C9" s="14" t="str">
-        <x:v>trained from scratch (historical)</x:v>
+        <x:v>retrained on development (historical)</x:v>
       </x:c>
       <x:c r="D9" s="14" t="str">
         <x:v>held-out test</x:v>
@@ -798,8 +823,8 @@
       <x:c r="M1" s="1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="3" t="s">
-        <x:v>15</x:v>
+      <x:c r="A2" s="3" t="str">
+        <x:v>Historical SAT and TreeX site metrics. Final SAT target aggregates are in Results Summary; retained Barkla files support future site aggregation.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -825,7 +850,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
         <x:v>5</x:v>
@@ -857,7 +882,7 @@
     </x:row>
     <x:row r="6" ht="16">
       <x:c r="A6" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
         <x:v>SegmentAnyTree (historical from-scratch)</x:v>
@@ -898,7 +923,7 @@
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
         <x:v>SegmentAnyTree (historical from-scratch)</x:v>
@@ -939,7 +964,7 @@
     </x:row>
     <x:row r="8" ht="16">
       <x:c r="A8" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
         <x:v>SegmentAnyTree (historical from-scratch)</x:v>
@@ -980,7 +1005,7 @@
     </x:row>
     <x:row r="9" ht="16">
       <x:c r="A9" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
         <x:v>SegmentAnyTree (historical from-scratch)</x:v>
@@ -1021,7 +1046,7 @@
     </x:row>
     <x:row r="10" ht="16">
       <x:c r="A10" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
         <x:v>SegmentAnyTree (historical from-scratch)</x:v>
@@ -1062,7 +1087,7 @@
     </x:row>
     <x:row r="11" ht="16">
       <x:c r="A11" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
         <x:v>TreeX</x:v>
@@ -1103,7 +1128,7 @@
     </x:row>
     <x:row r="12" ht="16">
       <x:c r="A12" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
         <x:v>TreeX</x:v>
@@ -1144,7 +1169,7 @@
     </x:row>
     <x:row r="13" ht="16">
       <x:c r="A13" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
         <x:v>TreeX</x:v>
@@ -1185,7 +1210,7 @@
     </x:row>
     <x:row r="14" ht="16">
       <x:c r="A14" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
         <x:v>TreeX</x:v>
@@ -1226,7 +1251,7 @@
     </x:row>
     <x:row r="15" ht="16">
       <x:c r="A15" s="5" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
         <x:v>TreeX</x:v>
@@ -1411,7 +1436,7 @@
   <x:sheetData>
     <x:row r="1" ht="20">
       <x:c r="A1" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -1419,7 +1444,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1427,25 +1452,25 @@
     </x:row>
     <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="D5" s="8" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="s">
+      <x:c r="E5" s="8" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="E5" s="8" t="s">
+      <x:c r="F5" s="8" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="s">
+      <x:c r="G5" s="8" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="G5" s="8" t="s">
+      <x:c r="H5" s="8" t="s">
         <x:v>25</x:v>
-      </x:c>
-      <x:c r="H5" s="8" t="s">
-        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
@@ -1453,10 +1478,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="D6" t="s">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="D6" t="s">
-        <x:v>28</x:v>
       </x:c>
       <x:c r="E6">
         <x:v>1</x:v>
@@ -1473,13 +1498,13 @@
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="s">
+      <x:c r="D7" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="D7" t="s">
-        <x:v>31</x:v>
       </x:c>
       <x:c r="E7">
         <x:v>11</x:v>
@@ -1499,10 +1524,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="D8" t="s">
         <x:v>32</x:v>
-      </x:c>
-      <x:c r="D8" t="s">
-        <x:v>33</x:v>
       </x:c>
       <x:c r="E8">
         <x:v>1</x:v>
@@ -1522,10 +1547,10 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>Current target: aligned released-checkpoint test, then released-weight fine-tuning on development data and aligned test. The completed from-scratch result (mean plot F1 0.4825; micro F1 0.4692) remains historical.</x:v>
+        <x:v>Completed primary: released-weight fine-tune mean plot F1 0.5447 and micro F1 0.5320. Published baseline mean plot F1 0.4534 and micro F1 0.4442. Historical retrained mean plot F1 0.4825 and micro F1 0.4692. Final target site rows are not shown because their per-plot table has not been transferred locally; aligned Barkla predictions are retained for future aggregation.</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E9">
         <x:v>3</x:v>
@@ -1548,7 +1573,7 @@
         <x:v>TreeX remains the completed deterministic baseline. Corrected union-mask test mean plot F1 is 0.3831 and micro F1 is 0.3627.</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E10">
         <x:v>0</x:v>
@@ -1567,7 +1592,7 @@
       <x:c r="A11" s="5"/>
       <x:c r="B11" s="5"/>
       <x:c r="D11" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E11" s="8">
         <x:v>16</x:v>
@@ -1613,7 +1638,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="D15" s="8" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E15" s="8" t="s">
         <x:v>5</x:v>
@@ -1624,7 +1649,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="D16" t="s">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="E16">
         <x:v>21</x:v>
@@ -1635,7 +1660,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="D17" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E17">
         <x:v>11</x:v>
@@ -1646,7 +1671,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="D18" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E18">
         <x:v>32</x:v>

</xml_diff>

<commit_message>
Record SegmentAnyTree site results
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R230dab76ef3e4539"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Ra66e0dfcd851485b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="R03da0b1830544b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R90a91aac2e3f476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R64d830f9099f447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" r:id="Rc22d0ff76aea464f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,12 +57,6 @@
     <x:t xml:space="preserve">FOR-instance Site Breakdown</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Site</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FOR-instance</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Notes</x:t>
   </x:si>
   <x:si>
@@ -127,9 +121,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="164" formatCode="0.000"/>
     <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -173,7 +168,7 @@
       <x:patternFill patternType="gray125"/>
     </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="5">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -203,11 +198,39 @@
         <x:color rgb="FFD9E2F3"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C7E7"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -239,11 +262,63 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SiteBreakdownTable" displayName="SiteBreakdownTable" ref="A5:M25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Dataset"/>
+    <x:tableColumn id="2" name="Method"/>
+    <x:tableColumn id="3" name="Evaluation split"/>
+    <x:tableColumn id="4" name="Site"/>
+    <x:tableColumn id="5" name="Plots"/>
+    <x:tableColumn id="6" name="F1 (IoU &gt;= 0.5)"/>
+    <x:tableColumn id="7" name="Precision"/>
+    <x:tableColumn id="8" name="Recall"/>
+    <x:tableColumn id="9" name="Mean segment IoU"/>
+    <x:tableColumn id="10" name="TP"/>
+    <x:tableColumn id="11" name="FP"/>
+    <x:tableColumn id="12" name="FN"/>
+    <x:tableColumn id="13" name="Brief note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -790,19 +865,21 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.6640625" style="2" customWidth="1"/>
-    <x:col min="2" max="2" width="15.33203125" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="14.83203125" style="2" customWidth="1"/>
-    <x:col min="4" max="4" width="8.33203125" style="2" customWidth="1"/>
-    <x:col min="5" max="5" width="5.6640625" style="2" customWidth="1"/>
-    <x:col min="6" max="6" width="13.6640625" style="2" customWidth="1"/>
-    <x:col min="7" max="7" width="9.33203125" style="2" customWidth="1"/>
-    <x:col min="8" max="8" width="6.5" style="2" customWidth="1"/>
-    <x:col min="9" max="9" width="14" style="2" customWidth="1"/>
+    <x:col min="1" max="1" width="15.779999732971191" style="2" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28.329999923706055" style="2" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18.670000076293945" style="2" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10.4399995803833" style="2" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.110000133514404" style="2" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17.110000610351562" style="2" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.779999732971191" style="2" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10.220000267028809" style="2" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.559999465942383" style="2" hidden="0" customWidth="1"/>
     <x:col min="10" max="11" width="4.1640625" style="2" customWidth="1"/>
-    <x:col min="12" max="12" width="3.6640625" style="2" customWidth="1"/>
-    <x:col min="13" max="13" width="61.83203125" style="2" customWidth="1"/>
+    <x:col min="12" max="12" width="5.329999923706055" style="2" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="56.66999816894531" style="2" hidden="0" customWidth="1"/>
     <x:col min="14" max="16384" width="8.83203125" style="2" customWidth="0"/>
+    <x:col min="10" max="10" width="5.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="5.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="20">
@@ -824,7 +901,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>Historical SAT and TreeX site metrics. Final SAT target aggregates are in Results Summary; retained Barkla files support future site aggregation.</x:v>
+        <x:v>Completed SAT target, historical SAT and TreeX site metrics. F1, precision and recall are site means; counts are summed.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -840,575 +917,865 @@
       <x:c r="M2" s="3"/>
     </x:row>
     <x:row r="5" ht="32">
-      <x:c r="A5" s="4" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="A5" s="4" t="str">
+        <x:v>Dataset</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="str">
+        <x:v>Evaluation split</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="str">
+        <x:v>Plots</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>F1 (IoU &gt;= 0.5)</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="str">
+        <x:v>Precision</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="I5" s="4" t="str">
+        <x:v>Mean segment IoU</x:v>
+      </x:c>
+      <x:c r="J5" s="4" t="str">
+        <x:v>TP</x:v>
+      </x:c>
+      <x:c r="K5" s="4" t="str">
+        <x:v>FP</x:v>
+      </x:c>
+      <x:c r="L5" s="4" t="str">
+        <x:v>FN</x:v>
+      </x:c>
+      <x:c r="M5" s="4" t="str">
+        <x:v>Brief note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="31.5" customHeight="1">
+      <x:c r="A6" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>SegmentAnyTree published pretrained (completed baseline)</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E6" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="n">
+        <x:v>0.45454545454545453</x:v>
+      </x:c>
+      <x:c r="G6" s="20" t="n">
+        <x:v>0.29411764705882354</x:v>
+      </x:c>
+      <x:c r="H6" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I6" s="20" t="n">
+        <x:v>0.976602030863474</x:v>
+      </x:c>
+      <x:c r="J6" s="19" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K6" s="19" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="L6" s="19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="13" t="str">
+        <x:v>Completed baseline site result; micro F1 0.4545.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="31.5" customHeight="1">
+      <x:c r="A7" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>SegmentAnyTree published pretrained (completed baseline)</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E7" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="n">
+        <x:v>0.4262686942306885</x:v>
+      </x:c>
+      <x:c r="G7" s="20" t="n">
+        <x:v>0.28840417589052403</x:v>
+      </x:c>
+      <x:c r="H7" s="20" t="n">
+        <x:v>0.8381366955928359</x:v>
+      </x:c>
+      <x:c r="I7" s="20" t="n">
+        <x:v>0.8587615056225794</x:v>
+      </x:c>
+      <x:c r="J7" s="19" t="n">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="K7" s="19" t="n">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="L7" s="19" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="M7" s="13" t="str">
+        <x:v>Completed baseline site result; micro F1 0.4290.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="31.5" customHeight="1">
+      <x:c r="A8" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>SegmentAnyTree published pretrained (completed baseline)</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G8" s="20" t="n">
+        <x:v>0.4318181818181818</x:v>
+      </x:c>
+      <x:c r="H8" s="20" t="n">
+        <x:v>0.59375</x:v>
+      </x:c>
+      <x:c r="I8" s="20" t="n">
+        <x:v>0.8165401196293979</x:v>
+      </x:c>
+      <x:c r="J8" s="19" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="K8" s="19" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="L8" s="19" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="M8" s="13" t="str">
+        <x:v>Completed baseline site result; micro F1 0.5000.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="31.5" customHeight="1">
+      <x:c r="A9" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>SegmentAnyTree published pretrained (completed baseline)</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E9" s="19" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="F9" s="20" t="n">
+        <x:v>0.5856705762366139</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="n">
+        <x:v>0.44285714285714284</x:v>
+      </x:c>
+      <x:c r="H9" s="20" t="n">
+        <x:v>0.8644444444444443</x:v>
+      </x:c>
+      <x:c r="I9" s="20" t="n">
+        <x:v>0.9009275764810685</x:v>
+      </x:c>
+      <x:c r="J9" s="19" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="K9" s="19" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="L9" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="M9" s="13" t="str">
+        <x:v>Completed baseline site result; micro F1 0.5827.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="31.5" customHeight="1">
+      <x:c r="A10" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>SegmentAnyTree published pretrained (completed baseline)</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E10" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="20" t="n">
+        <x:v>0.304</x:v>
+      </x:c>
+      <x:c r="G10" s="20" t="n">
+        <x:v>0.2111111111111111</x:v>
+      </x:c>
+      <x:c r="H10" s="20" t="n">
+        <x:v>0.5428571428571428</x:v>
+      </x:c>
+      <x:c r="I10" s="20" t="n">
+        <x:v>0.7157372006258339</x:v>
+      </x:c>
+      <x:c r="J10" s="19" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="K10" s="19" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L10" s="19" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="M10" s="13" t="str">
+        <x:v>Completed baseline site result; micro F1 0.3040.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="31.5" customHeight="1">
+      <x:c r="A11" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>SegmentAnyTree fine-tuned on development (primary)</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E11" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F11" s="20" t="n">
+        <x:v>0.49382716049382713</x:v>
+      </x:c>
+      <x:c r="G11" s="20" t="n">
+        <x:v>0.32786885245901637</x:v>
+      </x:c>
+      <x:c r="H11" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I11" s="20" t="n">
+        <x:v>0.9874771324959299</x:v>
+      </x:c>
+      <x:c r="J11" s="19" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K11" s="19" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="L11" s="19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="13" t="str">
+        <x:v>Primary site result; mean F1 +0.0393 vs released baseline; micro F1 0.4938.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="31.5" customHeight="1">
+      <x:c r="A12" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>SegmentAnyTree fine-tuned on development (primary)</x:v>
+      </x:c>
+      <x:c r="C12" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D12" s="17" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E12" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F12" s="20" t="n">
+        <x:v>0.5355587555717329</x:v>
+      </x:c>
+      <x:c r="G12" s="20" t="n">
+        <x:v>0.4042784369436756</x:v>
+      </x:c>
+      <x:c r="H12" s="20" t="n">
+        <x:v>0.8072796480691218</x:v>
+      </x:c>
+      <x:c r="I12" s="20" t="n">
+        <x:v>0.854806108122465</x:v>
+      </x:c>
+      <x:c r="J12" s="19" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="K12" s="19" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="L12" s="19" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="M12" s="13" t="str">
+        <x:v>Primary site result; mean F1 +0.1093 vs released baseline; micro F1 0.5375.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="31.5" customHeight="1">
+      <x:c r="A13" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>SegmentAnyTree fine-tuned on development (primary)</x:v>
+      </x:c>
+      <x:c r="C13" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D13" s="17" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E13" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F13" s="20" t="n">
+        <x:v>0.4768211920529801</x:v>
+      </x:c>
+      <x:c r="G13" s="20" t="n">
+        <x:v>0.41379310344827586</x:v>
+      </x:c>
+      <x:c r="H13" s="20" t="n">
+        <x:v>0.5625</x:v>
+      </x:c>
+      <x:c r="I13" s="20" t="n">
+        <x:v>0.7956887469952446</x:v>
+      </x:c>
+      <x:c r="J13" s="19" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="K13" s="19" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="L13" s="19" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="M13" s="13" t="str">
+        <x:v>Primary site result; mean F1 -0.0232 vs released baseline; micro F1 0.4768.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="31.5" customHeight="1">
+      <x:c r="A14" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>SegmentAnyTree fine-tuned on development (primary)</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D14" s="17" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E14" s="19" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="20" t="n">
+        <x:v>0.7206349206349205</x:v>
+      </x:c>
+      <x:c r="G14" s="20" t="n">
+        <x:v>0.5989278752436646</x:v>
+      </x:c>
+      <x:c r="H14" s="20" t="n">
+        <x:v>0.9044444444444444</x:v>
+      </x:c>
+      <x:c r="I14" s="20" t="n">
+        <x:v>0.9139943500562222</x:v>
+      </x:c>
+      <x:c r="J14" s="19" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="K14" s="19" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="L14" s="19" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
+      <x:c r="M14" s="13" t="str">
+        <x:v>Primary site result; mean F1 +0.1350 vs released baseline; micro F1 0.7222.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="31.5" customHeight="1">
+      <x:c r="A15" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B15" s="17" t="str">
+        <x:v>SegmentAnyTree fine-tuned on development (primary)</x:v>
+      </x:c>
+      <x:c r="C15" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D15" s="17" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E15" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F15" s="20" t="n">
+        <x:v>0.3661971830985915</x:v>
+      </x:c>
+      <x:c r="G15" s="20" t="n">
+        <x:v>0.3611111111111111</x:v>
+      </x:c>
+      <x:c r="H15" s="20" t="n">
+        <x:v>0.37142857142857144</x:v>
+      </x:c>
+      <x:c r="I15" s="20" t="n">
+        <x:v>0.7031941065901006</x:v>
+      </x:c>
+      <x:c r="J15" s="19" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="K15" s="19" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L15" s="19" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="M15" s="13" t="str">
+        <x:v>Primary site result; mean F1 +0.0622 vs released baseline; micro F1 0.3662.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="31.5" customHeight="1">
+      <x:c r="A16" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B16" s="17" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C16" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D16" s="17" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E16" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F16" s="20" t="n">
+        <x:v>0.5479452054794521</x:v>
+      </x:c>
+      <x:c r="G16" s="20" t="n">
+        <x:v>0.37735849056603776</x:v>
+      </x:c>
+      <x:c r="H16" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" s="20" t="n">
+        <x:v>0.9476273064944747</x:v>
+      </x:c>
+      <x:c r="J16" s="19" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K16" s="19" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="L16" s="19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M16" s="13" t="str">
+        <x:v>Historical site result; retained for traceability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="31.5" customHeight="1">
+      <x:c r="A17" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B17" s="17" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C17" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D17" s="17" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E17" s="19" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H5" s="4" t="s">
+      <x:c r="F17" s="20" t="n">
+        <x:v>0.47905399926507836</x:v>
+      </x:c>
+      <x:c r="G17" s="20" t="n">
+        <x:v>0.36172209807653116</x:v>
+      </x:c>
+      <x:c r="H17" s="20" t="n">
+        <x:v>0.7215901365024172</x:v>
+      </x:c>
+      <x:c r="I17" s="20" t="n">
+        <x:v>0.8395179520359185</x:v>
+      </x:c>
+      <x:c r="J17" s="19" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="K17" s="19" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="L17" s="19" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="M17" s="13" t="str">
+        <x:v>Historical site result; high recall with many false positives.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="31.5" customHeight="1">
+      <x:c r="A18" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B18" s="17" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C18" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D18" s="17" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E18" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="20" t="n">
+        <x:v>0.34426229508196726</x:v>
+      </x:c>
+      <x:c r="G18" s="20" t="n">
+        <x:v>0.3620689655172414</x:v>
+      </x:c>
+      <x:c r="H18" s="20" t="n">
+        <x:v>0.328125</x:v>
+      </x:c>
+      <x:c r="I18" s="20" t="n">
+        <x:v>0.7782650555699895</x:v>
+      </x:c>
+      <x:c r="J18" s="19" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K18" s="19" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="L18" s="19" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="M18" s="13" t="str">
+        <x:v>Historical site result; weak transfer and low recall.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="31.5" customHeight="1">
+      <x:c r="A19" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C19" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D19" s="17" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E19" s="19" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F19" s="20" t="n">
+        <x:v>0.6430575035063114</x:v>
+      </x:c>
+      <x:c r="G19" s="20" t="n">
+        <x:v>0.5337837837837838</x:v>
+      </x:c>
+      <x:c r="H19" s="20" t="n">
+        <x:v>0.8088888888888889</x:v>
+      </x:c>
+      <x:c r="I19" s="20" t="n">
+        <x:v>0.9122697775138862</x:v>
+      </x:c>
+      <x:c r="J19" s="19" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="K19" s="19" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L19" s="19" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I5" s="4" t="s">
+      <x:c r="M19" s="13" t="str">
+        <x:v>Historical site result; strongest retained SAT site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="31.5" customHeight="1">
+      <x:c r="A20" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B20" s="17" t="str">
+        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
+      </x:c>
+      <x:c r="C20" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D20" s="17" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E20" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F20" s="20" t="n">
+        <x:v>0.22535211267605634</x:v>
+      </x:c>
+      <x:c r="G20" s="20" t="n">
+        <x:v>0.2222222222222222</x:v>
+      </x:c>
+      <x:c r="H20" s="20" t="n">
+        <x:v>0.22857142857142856</x:v>
+      </x:c>
+      <x:c r="I20" s="20" t="n">
+        <x:v>0.6416865043044996</x:v>
+      </x:c>
+      <x:c r="J20" s="19" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K20" s="19" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="L20" s="19" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="M20" s="13" t="str">
+        <x:v>Historical site result; weak transfer and low recall.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="31.5" customHeight="1">
+      <x:c r="A21" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B21" s="17" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C21" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D21" s="17" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="E21" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F21" s="20" t="n">
+        <x:v>0.5797101449275363</x:v>
+      </x:c>
+      <x:c r="G21" s="20" t="n">
+        <x:v>0.40816326530612246</x:v>
+      </x:c>
+      <x:c r="H21" s="20" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I21" s="20" t="n">
+        <x:v>0.9384354128263748</x:v>
+      </x:c>
+      <x:c r="J21" s="19" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K21" s="19" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="L21" s="19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M21" s="13" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="31.5" customHeight="1">
+      <x:c r="A22" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B22" s="17" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C22" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D22" s="17" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="E22" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F22" s="20" t="n">
+        <x:v>0.34632498065993217</x:v>
+      </x:c>
+      <x:c r="G22" s="20" t="n">
+        <x:v>0.23478260869565218</x:v>
+      </x:c>
+      <x:c r="H22" s="20" t="n">
+        <x:v>0.6708074534161491</x:v>
+      </x:c>
+      <x:c r="I22" s="20" t="n">
+        <x:v>0.7750563475089646</x:v>
+      </x:c>
+      <x:c r="J22" s="19" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="K22" s="19" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="L22" s="19" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="M22" s="13" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="31.5" customHeight="1">
+      <x:c r="A23" s="17" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B23" s="17" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C23" s="17" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D23" s="17" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="E23" s="19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F23" s="20" t="n">
+        <x:v>0.216867469879518</x:v>
+      </x:c>
+      <x:c r="G23" s="20" t="n">
+        <x:v>0.47368421052631576</x:v>
+      </x:c>
+      <x:c r="H23" s="20" t="n">
+        <x:v>0.140625</x:v>
+      </x:c>
+      <x:c r="I23" s="20" t="n">
+        <x:v>0.8964955219132982</x:v>
+      </x:c>
+      <x:c r="J23" s="19" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="J5" s="4" t="s">
+      <x:c r="K23" s="19" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K5" s="4" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="L5" s="4" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="M5" s="4" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="16">
-      <x:c r="A6" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B6" s="5" t="str">
-        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="str">
-        <x:v>CULS</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="n">
-        <x:v>0.5479452054794521</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="n">
-        <x:v>0.37735849056603776</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I6" s="7" t="n">
-        <x:v>0.9476273064944747</x:v>
-      </x:c>
-      <x:c r="J6" s="6" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K6" s="6" t="n">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="L6" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M6" s="5" t="str">
-        <x:v>Historical site result; retained for traceability.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="16">
-      <x:c r="A7" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="str">
-        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="str">
-        <x:v>NIBIO</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="F7" s="7" t="n">
-        <x:v>0.47905399926507836</x:v>
-      </x:c>
-      <x:c r="G7" s="7" t="n">
-        <x:v>0.36172209807653116</x:v>
-      </x:c>
-      <x:c r="H7" s="7" t="n">
-        <x:v>0.7215901365024172</x:v>
-      </x:c>
-      <x:c r="I7" s="7" t="n">
-        <x:v>0.8395179520359185</x:v>
-      </x:c>
-      <x:c r="J7" s="6" t="n">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="K7" s="6" t="n">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="L7" s="6" t="n">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="M7" s="5" t="str">
-        <x:v>Historical site result; high recall with many false positives.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="16">
-      <x:c r="A8" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="str">
-        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="str">
-        <x:v>RMIT</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F8" s="7" t="n">
-        <x:v>0.34426229508196726</x:v>
-      </x:c>
-      <x:c r="G8" s="7" t="n">
-        <x:v>0.3620689655172414</x:v>
-      </x:c>
-      <x:c r="H8" s="7" t="n">
-        <x:v>0.328125</x:v>
-      </x:c>
-      <x:c r="I8" s="7" t="n">
-        <x:v>0.7782650555699895</x:v>
-      </x:c>
-      <x:c r="J8" s="6" t="n">
+      <x:c r="L23" s="19" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="M23" s="13" t="str">
+        <x:v>Low baseline site result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="31.5" customHeight="1">
+      <x:c r="A24" s="18" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B24" s="23" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C24" s="18" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D24" s="18" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="E24" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F24" s="22" t="n">
+        <x:v>0.5401987353206865</x:v>
+      </x:c>
+      <x:c r="G24" s="22" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H24" s="22" t="n">
+        <x:v>0.6046511627906976</x:v>
+      </x:c>
+      <x:c r="I24" s="22" t="n">
+        <x:v>0.8094268084447702</x:v>
+      </x:c>
+      <x:c r="J24" s="21" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="L24" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="M24" s="14" t="str">
+        <x:v>Completed aligned point-wise baseline site result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="31.5" customHeight="1">
+      <x:c r="A25" s="18" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B25" s="23" t="str">
+        <x:v>TreeX</x:v>
+      </x:c>
+      <x:c r="C25" s="18" t="str">
+        <x:v>held-out test</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="E25" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F25" s="22" t="n">
+        <x:v>0.2592592592592592</x:v>
+      </x:c>
+      <x:c r="G25" s="22" t="n">
+        <x:v>0.1917808219178082</x:v>
+      </x:c>
+      <x:c r="H25" s="22" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="I25" s="22" t="n">
+        <x:v>0.7372842800514755</x:v>
+      </x:c>
+      <x:c r="J25" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="L25" s="21" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="K8" s="6" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="L8" s="6" t="n">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="M8" s="5" t="str">
-        <x:v>Historical site result; weak transfer and low recall.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="16">
-      <x:c r="A9" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="str">
-        <x:v>SCION</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F9" s="7" t="n">
-        <x:v>0.6430575035063114</x:v>
-      </x:c>
-      <x:c r="G9" s="7" t="n">
-        <x:v>0.5337837837837838</x:v>
-      </x:c>
-      <x:c r="H9" s="7" t="n">
-        <x:v>0.8088888888888889</x:v>
-      </x:c>
-      <x:c r="I9" s="7" t="n">
-        <x:v>0.9122697775138862</x:v>
-      </x:c>
-      <x:c r="J9" s="6" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="K9" s="6" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="L9" s="6" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="M9" s="5" t="str">
-        <x:v>Historical site result; strongest retained SAT site.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="16">
-      <x:c r="A10" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B10" s="5" t="str">
-        <x:v>SegmentAnyTree (historical from-scratch)</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="str">
-        <x:v>TUWIEN</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F10" s="7" t="n">
-        <x:v>0.22535211267605634</x:v>
-      </x:c>
-      <x:c r="G10" s="7" t="n">
-        <x:v>0.2222222222222222</x:v>
-      </x:c>
-      <x:c r="H10" s="7" t="n">
-        <x:v>0.22857142857142856</x:v>
-      </x:c>
-      <x:c r="I10" s="7" t="n">
-        <x:v>0.6416865043044996</x:v>
-      </x:c>
-      <x:c r="J10" s="6" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="K10" s="6" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="L10" s="6" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="M10" s="5" t="str">
-        <x:v>Historical site result; weak transfer and low recall.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="16">
-      <x:c r="A11" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B11" s="5" t="str">
-        <x:v>TreeX</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="str">
-        <x:v>CULS</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F11" s="7" t="n">
-        <x:v>0.5797101449275363</x:v>
-      </x:c>
-      <x:c r="G11" s="7" t="n">
-        <x:v>0.40816326530612246</x:v>
-      </x:c>
-      <x:c r="H11" s="7" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I11" s="7" t="n">
-        <x:v>0.9384354128263748</x:v>
-      </x:c>
-      <x:c r="J11" s="6" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K11" s="6" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="L11" s="6" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M11" s="5" t="str">
-        <x:v>Completed aligned point-wise baseline site result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="16">
-      <x:c r="A12" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B12" s="5" t="str">
-        <x:v>TreeX</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="str">
-        <x:v>NIBIO</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="F12" s="7" t="n">
-        <x:v>0.34632498065993217</x:v>
-      </x:c>
-      <x:c r="G12" s="7" t="n">
-        <x:v>0.23478260869565218</x:v>
-      </x:c>
-      <x:c r="H12" s="7" t="n">
-        <x:v>0.6708074534161491</x:v>
-      </x:c>
-      <x:c r="I12" s="7" t="n">
-        <x:v>0.7750563475089646</x:v>
-      </x:c>
-      <x:c r="J12" s="6" t="n">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="K12" s="6" t="n">
-        <x:v>352</x:v>
-      </x:c>
-      <x:c r="L12" s="6" t="n">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="M12" s="5" t="str">
-        <x:v>Completed aligned point-wise baseline site result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="16">
-      <x:c r="A13" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B13" s="5" t="str">
-        <x:v>TreeX</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D13" s="5" t="str">
-        <x:v>RMIT</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="n">
-        <x:v>0.216867469879518</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="n">
-        <x:v>0.47368421052631576</x:v>
-      </x:c>
-      <x:c r="H13" s="7" t="n">
-        <x:v>0.140625</x:v>
-      </x:c>
-      <x:c r="I13" s="7" t="n">
-        <x:v>0.8964955219132982</x:v>
-      </x:c>
-      <x:c r="J13" s="6" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="K13" s="6" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="L13" s="6" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="M13" s="5" t="str">
+      <x:c r="M25" s="14" t="str">
         <x:v>Low baseline site result.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="16">
-      <x:c r="A14" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="str">
-        <x:v>TreeX</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="str">
-        <x:v>SCION</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="n">
-        <x:v>0.5401987353206865</x:v>
-      </x:c>
-      <x:c r="G14" s="7" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="H14" s="7" t="n">
-        <x:v>0.6046511627906976</x:v>
-      </x:c>
-      <x:c r="I14" s="7" t="n">
-        <x:v>0.8094268084447702</x:v>
-      </x:c>
-      <x:c r="J14" s="6" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="K14" s="6" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="L14" s="6" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="M14" s="5" t="str">
-        <x:v>Completed aligned point-wise baseline site result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="16">
-      <x:c r="A15" s="5" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B15" s="5" t="str">
-        <x:v>TreeX</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="str">
-        <x:v>held-out test</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="str">
-        <x:v>TUWIEN</x:v>
-      </x:c>
-      <x:c r="E15" s="6" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="n">
-        <x:v>0.2592592592592592</x:v>
-      </x:c>
-      <x:c r="G15" s="7" t="n">
-        <x:v>0.1917808219178082</x:v>
-      </x:c>
-      <x:c r="H15" s="7" t="n">
-        <x:v>0.4</x:v>
-      </x:c>
-      <x:c r="I15" s="7" t="n">
-        <x:v>0.7372842800514755</x:v>
-      </x:c>
-      <x:c r="J15" s="6" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="K15" s="6" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="L15" s="6" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="M15" s="5" t="str">
-        <x:v>Low baseline site result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="16">
-      <x:c r="A16" s="5"/>
-      <x:c r="B16" s="5"/>
-      <x:c r="C16" s="5"/>
-      <x:c r="D16" s="5"/>
-      <x:c r="E16" s="6"/>
-      <x:c r="F16" s="7"/>
-      <x:c r="G16" s="7"/>
-      <x:c r="H16" s="7"/>
-      <x:c r="I16" s="7"/>
-      <x:c r="J16" s="6"/>
-      <x:c r="K16" s="6"/>
-      <x:c r="L16" s="6"/>
-      <x:c r="M16" s="5"/>
-    </x:row>
-    <x:row r="17" ht="16">
-      <x:c r="A17" s="5"/>
-      <x:c r="B17" s="5"/>
-      <x:c r="C17" s="5"/>
-      <x:c r="D17" s="5"/>
-      <x:c r="E17" s="6"/>
-      <x:c r="F17" s="7"/>
-      <x:c r="G17" s="7"/>
-      <x:c r="H17" s="7"/>
-      <x:c r="I17" s="7"/>
-      <x:c r="J17" s="6"/>
-      <x:c r="K17" s="6"/>
-      <x:c r="L17" s="6"/>
-      <x:c r="M17" s="5"/>
-    </x:row>
-    <x:row r="18" ht="16">
-      <x:c r="A18" s="5"/>
-      <x:c r="B18" s="5"/>
-      <x:c r="C18" s="5"/>
-      <x:c r="D18" s="5"/>
-      <x:c r="E18" s="6"/>
-      <x:c r="F18" s="7"/>
-      <x:c r="G18" s="7"/>
-      <x:c r="H18" s="7"/>
-      <x:c r="I18" s="7"/>
-      <x:c r="J18" s="6"/>
-      <x:c r="K18" s="6"/>
-      <x:c r="L18" s="6"/>
-      <x:c r="M18" s="5"/>
-    </x:row>
-    <x:row r="19" ht="16">
-      <x:c r="A19" s="5"/>
-      <x:c r="B19" s="5"/>
-      <x:c r="C19" s="5"/>
-      <x:c r="D19" s="5"/>
-      <x:c r="E19" s="6"/>
-      <x:c r="F19" s="7"/>
-      <x:c r="G19" s="7"/>
-      <x:c r="H19" s="7"/>
-      <x:c r="I19" s="7"/>
-      <x:c r="J19" s="6"/>
-      <x:c r="K19" s="6"/>
-      <x:c r="L19" s="6"/>
-      <x:c r="M19" s="5"/>
-    </x:row>
-    <x:row r="20" ht="16">
-      <x:c r="A20" s="5"/>
-      <x:c r="B20" s="5"/>
-      <x:c r="C20" s="5"/>
-      <x:c r="D20" s="5"/>
-      <x:c r="E20" s="6"/>
-      <x:c r="F20" s="7"/>
-      <x:c r="G20" s="7"/>
-      <x:c r="H20" s="7"/>
-      <x:c r="I20" s="7"/>
-      <x:c r="J20" s="6"/>
-      <x:c r="K20" s="6"/>
-      <x:c r="L20" s="6"/>
-      <x:c r="M20" s="5"/>
-    </x:row>
-    <x:row r="21" ht="16">
-      <x:c r="A21" s="5"/>
-      <x:c r="B21" s="5"/>
-      <x:c r="C21" s="5"/>
-      <x:c r="D21" s="5"/>
-      <x:c r="E21" s="6"/>
-      <x:c r="F21" s="7"/>
-      <x:c r="G21" s="7"/>
-      <x:c r="H21" s="7"/>
-      <x:c r="I21" s="7"/>
-      <x:c r="J21" s="6"/>
-      <x:c r="K21" s="6"/>
-      <x:c r="L21" s="6"/>
-      <x:c r="M21" s="5"/>
-    </x:row>
-    <x:row r="22" ht="16">
-      <x:c r="A22" s="5"/>
-      <x:c r="B22" s="5"/>
-      <x:c r="C22" s="5"/>
-      <x:c r="D22" s="5"/>
-      <x:c r="E22" s="6"/>
-      <x:c r="F22" s="7"/>
-      <x:c r="G22" s="7"/>
-      <x:c r="H22" s="7"/>
-      <x:c r="I22" s="7"/>
-      <x:c r="J22" s="6"/>
-      <x:c r="K22" s="6"/>
-      <x:c r="L22" s="6"/>
-      <x:c r="M22" s="5"/>
-    </x:row>
-    <x:row r="23" ht="16">
-      <x:c r="A23" s="5"/>
-      <x:c r="B23" s="5"/>
-      <x:c r="C23" s="5"/>
-      <x:c r="D23" s="5"/>
-      <x:c r="E23" s="6"/>
-      <x:c r="F23" s="7"/>
-      <x:c r="G23" s="7"/>
-      <x:c r="H23" s="7"/>
-      <x:c r="I23" s="7"/>
-      <x:c r="J23" s="6"/>
-      <x:c r="K23" s="6"/>
-      <x:c r="L23" s="6"/>
-      <x:c r="M23" s="5"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1416,6 +1783,9 @@
     <x:mergeCell ref="A2:M2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf05ebeac328e444f"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -1436,7 +1806,7 @@
   <x:sheetData>
     <x:row r="1" ht="20">
       <x:c r="A1" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -1444,7 +1814,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1452,25 +1822,25 @@
     </x:row>
     <x:row r="5" ht="16">
       <x:c r="A5" s="4" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="E5" s="8" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D5" s="8" t="s">
+      <x:c r="F5" s="8" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="E5" s="8" t="s">
+      <x:c r="G5" s="8" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="s">
+      <x:c r="H5" s="8" t="s">
         <x:v>23</x:v>
-      </x:c>
-      <x:c r="G5" s="8" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="H5" s="8" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16">
@@ -1478,10 +1848,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>26</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D6" t="s">
-        <x:v>27</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E6">
         <x:v>1</x:v>
@@ -1498,13 +1868,13 @@
     </x:row>
     <x:row r="7" ht="16">
       <x:c r="A7" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B7" s="5" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D7" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="B7" s="5" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D7" t="s">
-        <x:v>30</x:v>
       </x:c>
       <x:c r="E7">
         <x:v>11</x:v>
@@ -1524,10 +1894,10 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D8" t="s">
-        <x:v>32</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E8">
         <x:v>1</x:v>
@@ -1546,11 +1916,11 @@
       <x:c r="A9" s="5" t="str">
         <x:v>SegmentAnyTree</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="str">
-        <x:v>Completed primary: released-weight fine-tune mean plot F1 0.5447 and micro F1 0.5320. Published baseline mean plot F1 0.4534 and micro F1 0.4442. Historical retrained mean plot F1 0.4825 and micro F1 0.4692. Final target site rows are not shown because their per-plot table has not been transferred locally; aligned Barkla predictions are retained for future aggregation.</x:v>
+      <x:c r="B9" s="13" t="str">
+        <x:v>Completed primary: released-weight fine-tune mean plot F1 0.5447 and micro F1 0.5320. Published baseline mean plot F1 0.4534 and micro F1 0.4442. Historical retrained mean plot F1 0.4825 and micro F1 0.4692. Completed target site rows are shown in Site Breakdown; SCION is strongest for the primary run (0.7206) and TUWIEN is weakest (0.3662). Aligned Barkla predictions remain retained for future metrics.</x:v>
       </x:c>
       <x:c r="D9" t="s">
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E9">
         <x:v>3</x:v>
@@ -1569,11 +1939,11 @@
       <x:c r="A10" s="5" t="str">
         <x:v>TreeX</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B10" s="13" t="str">
         <x:v>TreeX remains the completed deterministic baseline. Corrected union-mask test mean plot F1 is 0.3831 and micro F1 is 0.3627.</x:v>
       </x:c>
       <x:c r="D10" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E10">
         <x:v>0</x:v>
@@ -1589,10 +1959,14 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="5"/>
-      <x:c r="B11" s="5"/>
+      <x:c r="A11" s="24" t="str">
+        <x:v>Site source</x:v>
+      </x:c>
+      <x:c r="B11" s="25" t="str">
+        <x:v>methods/segmentanytree/examples/sat_completed_target_site_results_20260711.csv; generated from retained per-plot aligned metric JSONs without rerunning inference.</x:v>
+      </x:c>
       <x:c r="D11" s="8" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E11" s="8">
         <x:v>16</x:v>
@@ -1638,7 +2012,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="D15" s="8" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="E15" s="8" t="s">
         <x:v>5</x:v>
@@ -1649,7 +2023,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="D16" t="s">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E16">
         <x:v>21</x:v>
@@ -1660,7 +2034,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="D17" t="s">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E17">
         <x:v>11</x:v>
@@ -1671,7 +2045,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="D18" t="s">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E18">
         <x:v>32</x:v>

</xml_diff>

<commit_message>
feat(treelearn): add split-locked long fine-tune workflow
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R9b43106334ab4efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R4db42082a27d401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="3" r:id="Rf4d832425e394493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="R3a7eb3fc6e894a12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R7e3c311bc5954a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R8d92ff4148ad433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="3" r:id="R99f93a718a9e4890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Re45199b12664461f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -330,7 +330,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -340,7 +340,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1038,7 +1038,7 @@
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q8" s="42" t="str">
-        <x:v>Development diagnostic only; not comparable with held-out test rows.</x:v>
+        <x:v>Published-checkpoint development diagnostic with documented FOR-instance validation/test training overlap; excluded from leakage-free ranking and not comparable with held-out test rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
@@ -1089,7 +1089,7 @@
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q9" s="42" t="str">
-        <x:v>Directly comparable only with the TreeLearn fine-tuned validation row.</x:v>
+        <x:v>Comparable only with the inherited-overlap TreeLearn fine-tuned validation row; excluded from leakage-free ranking.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -1143,7 +1143,7 @@
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q10" s="49" t="str">
-        <x:v>Best mean-F1 fine-tuned checkpoint; rejected because it underperformed the matched published baseline.</x:v>
+        <x:v>Best mean-F1 checkpoint inherited documented FOR-instance overlap from its initial weights and was rejected because it underperformed the matched baseline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1161,7 +1161,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2a4899eb1744d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7581f2a272e745bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2305,7 +2305,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R400dc57755b648a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R929418fb228d47af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2721,7 +2721,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ce39229a7434a92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdea02f453ede4dfb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2915,7 +2915,7 @@
         <x:v>TreeLearn full development</x:v>
       </x:c>
       <x:c r="B6" s="38" t="str">
-        <x:v>The 21-plot published TreeLearn result is a development diagnostic. It must not be ranked against held-out-test rows.</x:v>
+        <x:v>The 21-plot TreeLearn result is a development diagnostic from the December 2024 checkpoint. That checkpoint has documented FOR-instance validation/test training overlap, so this row is excluded from leakage-free ranking.</x:v>
       </x:c>
       <x:c r="C6" s="38" t="str">
         <x:v>methods/treelearn/examples/treelearn_completed_development_results_20260712.csv</x:v>
@@ -2940,7 +2940,7 @@
         <x:v>TreeLearn fine-tuning</x:v>
       </x:c>
       <x:c r="B7" s="38" t="str">
-        <x:v>The fine-tuned result is compared only with the published checkpoint on the identical five internal-validation plots. Fine-tuning regressed and was rejected before test.</x:v>
+        <x:v>The earlier fine-tuned result is compared only with its matched internal-validation baseline. It inherits the same checkpoint overlap and was rejected before test. The replacement clean-checkpoint route remains development-only.</x:v>
       </x:c>
       <x:c r="C7" s="38" t="str">
         <x:v>methods/treelearn/examples/treelearn_finetune_validation_results_20260712.csv</x:v>
@@ -3092,7 +3092,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc21002c6cf1e4113"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc292865f8be0402b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record completed TreeLearn held-out benchmark
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="R7e3c311bc5954a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R8d92ff4148ad433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="3" r:id="R99f93a718a9e4890"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Re45199b12664461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results Summary" sheetId="1" r:id="Rd6a0ef720d504597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rd2db27fa11f046ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="3" r:id="R4f1af193e44c411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Rbc0b134de3364852"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -168,7 +168,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -319,6 +319,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -367,7 +370,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BenchmarkResults" displayName="BenchmarkResults" ref="A4:Q10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BenchmarkResults" displayName="BenchmarkResults" ref="A4:Q11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Dataset"/>
     <x:tableColumn id="2" name="Method"/>
@@ -392,7 +395,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SiteResults" displayName="SiteResults" ref="A4:N24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SiteResults" displayName="SiteResults" ref="A4:N29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Dataset"/>
     <x:tableColumn id="2" name="Method"/>
@@ -414,7 +417,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RetentionRegistry" displayName="RetentionRegistry" ref="A4:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RetentionRegistry" displayName="RetentionRegistry" ref="A4:J11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Method"/>
     <x:tableColumn id="2" name="Variant"/>
@@ -432,7 +435,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComparabilityNotes" displayName="ComparabilityNotes" ref="A4:C12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ComparabilityNotes" displayName="ComparabilityNotes" ref="A4:C13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Topic"/>
     <x:tableColumn id="2" name="Rule"/>
@@ -711,55 +714,55 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="27" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="D2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="E2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="F2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="G2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="H2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="I2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="J2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="K2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="L2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="M2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="N2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="O2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="P2" s="28" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
       <x:c r="Q2" s="29" t="str">
-        <x:v>Headline comparison uses the identical 11-plot held-out test split. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
+        <x:v>Headline comparison uses the identical 11-plot held-out test split, including the frozen TreeLearn fine-tuned result. TreeLearn development diagnostics are shown separately and are not ranked against test rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -998,47 +1001,47 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C8" s="38" t="str">
-        <x:v>published pretrained full development</x:v>
+        <x:v>fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D8" s="38" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E8" s="38" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="F8" s="39" t="n">
-        <x:v>21</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G8" s="40" t="n">
-        <x:v>0.5155705605170436</x:v>
+        <x:v>0.36468463620440583</x:v>
       </x:c>
       <x:c r="H8" s="40" t="n">
-        <x:v>0.5107604017216643</x:v>
+        <x:v>0.33192389006342493</x:v>
       </x:c>
       <x:c r="I8" s="40"/>
       <x:c r="J8" s="40" t="n">
-        <x:v>0.4158878504672897</x:v>
+        <x:v>0.2520064205457464</x:v>
       </x:c>
       <x:c r="K8" s="40" t="n">
-        <x:v>0.6617100371747212</x:v>
+        <x:v>0.48606811145510836</x:v>
       </x:c>
       <x:c r="L8" s="41" t="n">
-        <x:v>534</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="M8" s="41" t="n">
-        <x:v>750</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="N8" s="41" t="n">
-        <x:v>273</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="O8" s="38" t="str">
-        <x:v>completed_aligned_pointwise_development</x:v>
+        <x:v>completed_aligned_pointwise_test</x:v>
       </x:c>
       <x:c r="P8" s="38" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q8" s="42" t="str">
-        <x:v>Published-checkpoint development diagnostic with documented FOR-instance validation/test training overlap; excluded from leakage-free ranking and not comparable with held-out test rows.</x:v>
+        <x:v>Preregistered seed-42 epoch-35 checkpoint evaluated once on the identical 11-plot test split; all 55 prediction artefacts are hash-verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" hidden="0" customHeight="1">
@@ -1049,47 +1052,47 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C9" s="38" t="str">
-        <x:v>published pretrained matched validation baseline</x:v>
+        <x:v>published pretrained full development</x:v>
       </x:c>
       <x:c r="D9" s="38" t="str">
-        <x:v>Internal dev validation</x:v>
+        <x:v>Full development</x:v>
       </x:c>
       <x:c r="E9" s="38" t="str">
-        <x:v>treelearn_matched_internal_validation</x:v>
+        <x:v>treelearn_full_development_diagnostic</x:v>
       </x:c>
       <x:c r="F9" s="39" t="n">
-        <x:v>5</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G9" s="40" t="n">
-        <x:v>0.558769</x:v>
+        <x:v>0.5155705605170436</x:v>
       </x:c>
       <x:c r="H9" s="40" t="n">
-        <x:v>0.5475285171102662</x:v>
+        <x:v>0.5107604017216643</x:v>
       </x:c>
       <x:c r="I9" s="40"/>
       <x:c r="J9" s="40" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.4158878504672897</x:v>
       </x:c>
       <x:c r="K9" s="40" t="n">
-        <x:v>0.6990291262135923</x:v>
+        <x:v>0.6617100371747212</x:v>
       </x:c>
       <x:c r="L9" s="41" t="n">
-        <x:v>144</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="M9" s="41" t="n">
-        <x:v>176</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="N9" s="41" t="n">
-        <x:v>62</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="O9" s="38" t="str">
-        <x:v>completed_matched_development_validation</x:v>
+        <x:v>completed_aligned_pointwise_development</x:v>
       </x:c>
       <x:c r="P9" s="38" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q9" s="42" t="str">
-        <x:v>Comparable only with the inherited-overlap TreeLearn fine-tuned validation row; excluded from leakage-free ranking.</x:v>
+        <x:v>Published-checkpoint development diagnostic with documented FOR-instance validation/test training overlap; excluded from leakage-free ranking and not comparable with held-out test rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" hidden="0" customHeight="1">
@@ -1100,7 +1103,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C10" s="45" t="str">
-        <x:v>fine-tuned on development epoch 70</x:v>
+        <x:v>published pretrained matched validation baseline</x:v>
       </x:c>
       <x:c r="D10" s="45" t="str">
         <x:v>Internal dev validation</x:v>
@@ -1112,37 +1115,90 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="47" t="n">
-        <x:v>0.4905044251328631</x:v>
+        <x:v>0.558769</x:v>
       </x:c>
       <x:c r="H10" s="47" t="n">
-        <x:v>0.42138364779874216</x:v>
+        <x:v>0.5475285171102662</x:v>
       </x:c>
       <x:c r="I10" s="47" t="n">
-        <x:f>G10-G9</x:f>
-        <x:v>-0.06826457486713688</x:v>
+        <x:v>0.04319843948295632</x:v>
       </x:c>
       <x:c r="J10" s="47" t="n">
-        <x:v>0.3116279069767442</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="K10" s="47" t="n">
-        <x:v>0.6504854368932039</x:v>
+        <x:v>0.6990291262135923</x:v>
       </x:c>
       <x:c r="L10" s="48" t="n">
-        <x:v>134</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="M10" s="48" t="n">
-        <x:v>296</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="N10" s="48" t="n">
-        <x:v>72</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="O10" s="45" t="str">
-        <x:v>rejected_validation_regression</x:v>
+        <x:v>completed_matched_development_validation</x:v>
       </x:c>
       <x:c r="P10" s="45" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
       <x:c r="Q10" s="49" t="str">
+        <x:v>Comparable only with the inherited-overlap TreeLearn fine-tuned validation row; excluded from leakage-free ranking.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>fine-tuned on development epoch 70</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Internal dev validation</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>treelearn_matched_internal_validation</x:v>
+      </x:c>
+      <x:c r="F11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G11" t="n">
+        <x:v>0.4905044251328631</x:v>
+      </x:c>
+      <x:c r="H11" t="n">
+        <x:v>0.42138364779874216</x:v>
+      </x:c>
+      <x:c r="I11" t="n">
+        <x:f>G11-G10</x:f>
+        <x:v>-0.06826457486713688</x:v>
+      </x:c>
+      <x:c r="J11" t="n">
+        <x:v>0.3116279069767442</x:v>
+      </x:c>
+      <x:c r="K11" t="n">
+        <x:v>0.6504854368932039</x:v>
+      </x:c>
+      <x:c r="L11" t="n">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="M11" t="n">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="N11" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>rejected_validation_regression</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>retention_verified</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
         <x:v>Best mean-F1 checkpoint inherited documented FOR-instance overlap from its initial weights and was rejected because it underperformed the matched baseline.</x:v>
       </x:c>
     </x:row>
@@ -1161,7 +1217,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7581f2a272e745bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ba3b7c967cb4c85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1172,7 +1228,7 @@
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="8" hidden="0" customWidth="1"/>
@@ -2071,40 +2127,40 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C20" s="31" t="str">
-        <x:v>Published pretrained</x:v>
+        <x:v>Fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D20" s="31" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E20" s="31" t="str">
         <x:v>CULS</x:v>
       </x:c>
       <x:c r="F20" s="50" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="51" t="n">
-        <x:v>0.7150101419878296</x:v>
+        <x:v>0.5333333333333333</x:v>
       </x:c>
       <x:c r="H20" s="51" t="n">
-        <x:v>0.72</x:v>
+        <x:v>0.5333333333333333</x:v>
       </x:c>
       <x:c r="I20" s="51" t="n">
-        <x:v>0.5625</x:v>
+        <x:v>0.36363636363636365</x:v>
       </x:c>
       <x:c r="J20" s="51" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K20" s="52" t="n">
-        <x:v>27</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="L20" s="52" t="n">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="M20" s="52" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N20" s="31" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="O20" s="31"/>
       <x:c r="P20" s="31"/>
@@ -2118,40 +2174,40 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C21" s="31" t="str">
-        <x:v>Published pretrained</x:v>
+        <x:v>Fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D21" s="31" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E21" s="31" t="str">
         <x:v>NIBIO</x:v>
       </x:c>
       <x:c r="F21" s="50" t="n">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G21" s="51" t="n">
-        <x:v>0.44696480338087335</x:v>
+        <x:v>0.2975920251871735</x:v>
       </x:c>
       <x:c r="H21" s="51" t="n">
-        <x:v>0.4466615502686109</x:v>
+        <x:v>0.2931937172774869</x:v>
       </x:c>
       <x:c r="I21" s="51" t="n">
-        <x:v>0.32733408323959506</x:v>
+        <x:v>0.20388349514563106</x:v>
       </x:c>
       <x:c r="J21" s="51" t="n">
-        <x:v>0.7028985507246377</x:v>
+        <x:v>0.5217391304347826</x:v>
       </x:c>
       <x:c r="K21" s="52" t="n">
-        <x:v>291</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="L21" s="52" t="n">
-        <x:v>598</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="M21" s="52" t="n">
-        <x:v>123</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="N21" s="31" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="O21" s="31"/>
       <x:c r="P21" s="31"/>
@@ -2165,10 +2221,10 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C22" s="31" t="str">
-        <x:v>Published pretrained</x:v>
+        <x:v>Fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D22" s="31" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E22" s="31" t="str">
         <x:v>RMIT</x:v>
@@ -2177,28 +2233,28 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G22" s="51" t="n">
-        <x:v>0.5894736842105263</x:v>
+        <x:v>0.16216216216216214</x:v>
       </x:c>
       <x:c r="H22" s="51" t="n">
-        <x:v>0.5894736842105263</x:v>
+        <x:v>0.16216216216216217</x:v>
       </x:c>
       <x:c r="I22" s="51" t="n">
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.19148936170212766</x:v>
       </x:c>
       <x:c r="J22" s="51" t="n">
-        <x:v>0.5283018867924528</x:v>
+        <x:v>0.140625</x:v>
       </x:c>
       <x:c r="K22" s="52" t="n">
-        <x:v>84</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="L22" s="52" t="n">
-        <x:v>42</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="M22" s="52" t="n">
-        <x:v>75</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="N22" s="31" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="O22" s="31"/>
       <x:c r="P22" s="31"/>
@@ -2212,40 +2268,40 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C23" s="31" t="str">
-        <x:v>Published pretrained</x:v>
+        <x:v>Fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D23" s="31" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E23" s="31" t="str">
         <x:v>SCION</x:v>
       </x:c>
       <x:c r="F23" s="50" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G23" s="51" t="n">
-        <x:v>0.652892069171139</x:v>
+        <x:v>0.620663362561952</x:v>
       </x:c>
       <x:c r="H23" s="51" t="n">
-        <x:v>0.6464646464646465</x:v>
+        <x:v>0.6153846153846154</x:v>
       </x:c>
       <x:c r="I23" s="51" t="n">
-        <x:v>0.6037735849056604</x:v>
+        <x:v>0.5245901639344263</x:v>
       </x:c>
       <x:c r="J23" s="51" t="n">
-        <x:v>0.6956521739130435</x:v>
+        <x:v>0.7441860465116279</x:v>
       </x:c>
       <x:c r="K23" s="52" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L23" s="52" t="n">
-        <x:v>42</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="M23" s="52" t="n">
-        <x:v>28</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="N23" s="31" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="O23" s="31"/>
       <x:c r="P23" s="31"/>
@@ -2259,10 +2315,10 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="C24" s="54" t="str">
-        <x:v>Published pretrained</x:v>
+        <x:v>Fine-tuned on development long epoch 35</x:v>
       </x:c>
       <x:c r="D24" s="54" t="str">
-        <x:v>Full development</x:v>
+        <x:v>Held-out test</x:v>
       </x:c>
       <x:c r="E24" s="54" t="str">
         <x:v>TUWIEN</x:v>
@@ -2271,32 +2327,252 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G24" s="56" t="n">
-        <x:v>0.591304347826087</x:v>
+        <x:v>0.2891566265060241</x:v>
       </x:c>
       <x:c r="H24" s="56" t="n">
-        <x:v>0.591304347826087</x:v>
+        <x:v>0.2891566265060241</x:v>
       </x:c>
       <x:c r="I24" s="56" t="n">
-        <x:v>0.591304347826087</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="J24" s="56" t="n">
-        <x:v>0.591304347826087</x:v>
+        <x:v>0.34285714285714286</x:v>
       </x:c>
       <x:c r="K24" s="57" t="n">
-        <x:v>68</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L24" s="57" t="n">
-        <x:v>47</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="M24" s="57" t="n">
-        <x:v>47</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N24" s="54" t="str">
-        <x:v>treelearn_full_development_diagnostic</x:v>
+        <x:v>held_out_test_primary</x:v>
       </x:c>
       <x:c r="O24" s="54"/>
       <x:c r="P24" s="54"/>
       <x:c r="Q24" s="58"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Published pretrained</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Full development</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>CULS</x:v>
+      </x:c>
+      <x:c r="F25" s="8" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G25" s="7" t="n">
+        <x:v>0.7150101419878296</x:v>
+      </x:c>
+      <x:c r="H25" s="7" t="n">
+        <x:v>0.72</x:v>
+      </x:c>
+      <x:c r="I25" s="7" t="n">
+        <x:v>0.5625</x:v>
+      </x:c>
+      <x:c r="J25" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K25" s="9" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="L25" s="9" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M25" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N25" t="str">
+        <x:v>treelearn_full_development_diagnostic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Published pretrained</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Full development</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>NIBIO</x:v>
+      </x:c>
+      <x:c r="F26" s="8" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G26" s="7" t="n">
+        <x:v>0.44696480338087335</x:v>
+      </x:c>
+      <x:c r="H26" s="7" t="n">
+        <x:v>0.4466615502686109</x:v>
+      </x:c>
+      <x:c r="I26" s="7" t="n">
+        <x:v>0.32733408323959506</x:v>
+      </x:c>
+      <x:c r="J26" s="7" t="n">
+        <x:v>0.7028985507246377</x:v>
+      </x:c>
+      <x:c r="K26" s="9" t="n">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="n">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="M26" s="9" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="N26" t="str">
+        <x:v>treelearn_full_development_diagnostic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Published pretrained</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Full development</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>RMIT</x:v>
+      </x:c>
+      <x:c r="F27" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G27" s="7" t="n">
+        <x:v>0.5894736842105263</x:v>
+      </x:c>
+      <x:c r="H27" s="7" t="n">
+        <x:v>0.5894736842105263</x:v>
+      </x:c>
+      <x:c r="I27" s="7" t="n">
+        <x:v>0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="J27" s="7" t="n">
+        <x:v>0.5283018867924528</x:v>
+      </x:c>
+      <x:c r="K27" s="9" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="L27" s="9" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M27" s="9" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="N27" t="str">
+        <x:v>treelearn_full_development_diagnostic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Published pretrained</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Full development</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>SCION</x:v>
+      </x:c>
+      <x:c r="F28" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G28" s="7" t="n">
+        <x:v>0.652892069171139</x:v>
+      </x:c>
+      <x:c r="H28" s="7" t="n">
+        <x:v>0.6464646464646465</x:v>
+      </x:c>
+      <x:c r="I28" s="7" t="n">
+        <x:v>0.6037735849056604</x:v>
+      </x:c>
+      <x:c r="J28" s="7" t="n">
+        <x:v>0.6956521739130435</x:v>
+      </x:c>
+      <x:c r="K28" s="9" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="M28" s="9" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="N28" t="str">
+        <x:v>treelearn_full_development_diagnostic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>FOR-instance</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Published pretrained</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Full development</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>TUWIEN</x:v>
+      </x:c>
+      <x:c r="F29" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G29" s="7" t="n">
+        <x:v>0.591304347826087</x:v>
+      </x:c>
+      <x:c r="H29" s="7" t="n">
+        <x:v>0.591304347826087</x:v>
+      </x:c>
+      <x:c r="I29" s="7" t="n">
+        <x:v>0.591304347826087</x:v>
+      </x:c>
+      <x:c r="J29" s="7" t="n">
+        <x:v>0.591304347826087</x:v>
+      </x:c>
+      <x:c r="K29" s="9" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="L29" s="9" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="M29" s="9" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="N29" t="str">
+        <x:v>treelearn_full_development_diagnostic</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2305,7 +2581,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R929418fb228d47af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6b2bf35fe8d47c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2714,6 +2990,36 @@
       <x:c r="P10" s="54"/>
       <x:c r="Q10" s="58"/>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>TreeLearn</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>fine_tuned_on_dev_long_epoch_35</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>treelearn_for-instance_fine_tuned_on_dev_long_20260712_233227</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>raw_and_aligned_predictions</x:v>
+      </x:c>
+      <x:c r="F11" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G11"/>
+      <x:c r="H11" t="str">
+        <x:v>sha256_verified</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>barkla_run_scoped_retained</x:v>
+      </x:c>
+      <x:c r="J11" s="22" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
@@ -2721,7 +3027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdea02f453ede4dfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra90fee945a1e440f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2890,7 +3196,7 @@
         <x:v>Headline comparison</x:v>
       </x:c>
       <x:c r="B5" s="38" t="str">
-        <x:v>SegmentAnyTree published, SegmentAnyTree fine-tuned and TreeX use the identical 11-plot held-out test split and shared harmonised evaluator.</x:v>
+        <x:v>SegmentAnyTree published, SegmentAnyTree fine-tuned, TreeX and the frozen TreeLearn epoch-35 result use the identical 11-plot test split, 323 references and shared evaluator.</x:v>
       </x:c>
       <x:c r="C5" s="38" t="str">
         <x:v>docs/protocols/for-instance.md</x:v>
@@ -2940,7 +3246,7 @@
         <x:v>TreeLearn fine-tuning</x:v>
       </x:c>
       <x:c r="B7" s="38" t="str">
-        <x:v>The earlier fine-tuned result is compared only with its matched internal-validation baseline. It inherits the same checkpoint overlap and was rejected before test. The replacement clean-checkpoint route remains development-only.</x:v>
+        <x:v>The earlier fine-tuned result is compared only with its matched internal-validation baseline. It inherits the December 2024 checkpoint overlap and was rejected before test. The separate clean-checkpoint epoch-35 route completed its one-time test and is recorded as a primary row.</x:v>
       </x:c>
       <x:c r="C7" s="38" t="str">
         <x:v>methods/treelearn/examples/treelearn_finetune_validation_results_20260712.csv</x:v>
@@ -3085,6 +3391,17 @@
       <x:c r="P12" s="54"/>
       <x:c r="Q12" s="58"/>
     </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="65" t="str">
+        <x:v>TreeLearn fine-tuned held-out test</x:v>
+      </x:c>
+      <x:c r="B13" s="65" t="str">
+        <x:v>The seed-42 epoch-35 checkpoint was frozen before its one-time 11-plot test. It is a primary comparable row; the published-checkpoint development diagnostic remains separate because of documented training overlap.</x:v>
+      </x:c>
+      <x:c r="C13" s="65" t="str">
+        <x:v>methods/treelearn/examples/treelearn_finetuned_test_results_20260713.csv</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:Q1"/>
@@ -3092,7 +3409,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc292865f8be0402b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R156deeee3de84b61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Reconcile public FOR-instance evidence
</commit_message>
<xml_diff>
--- a/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
+++ b/outputs/sat_treex_benchmark_metrics/for_instance_method_benchmark_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="R4c38b0a697364a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="R7cda3c0094f74297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="Rf9df49bd632f4ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Rc9da45f320cc4d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Results" sheetId="1" r:id="R22145fb569594b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Site Breakdown" sheetId="2" r:id="Rff045f0d69124541"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol Alignment" sheetId="3" r:id="Rff179ee13d3241ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction Retention" sheetId="4" r:id="Ra632d449caf04fc7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -432,9 +432,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.889999866485596" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12.779999732971191" hidden="0" customWidth="1"/>
@@ -551,7 +551,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>external_training_only</x:v>
@@ -659,7 +659,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>fine_tuned_on_dev</x:v>
@@ -767,7 +767,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
         <x:v>fine_tuned_on_dev</x:v>
@@ -823,7 +823,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R859dbeb4d1b54dbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R057079016a6b4280"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -832,9 +832,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="7.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12.779999732971191" hidden="0" customWidth="1"/>
@@ -933,7 +933,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>test</x:v>
@@ -977,7 +977,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
         <x:v>test</x:v>
@@ -1021,7 +1021,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>test</x:v>
@@ -1065,7 +1065,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
         <x:v>test</x:v>
@@ -1109,7 +1109,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
         <x:v>test</x:v>
@@ -1373,7 +1373,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
         <x:v>test</x:v>
@@ -1417,7 +1417,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
         <x:v>test</x:v>
@@ -1461,7 +1461,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
         <x:v>test</x:v>
@@ -1505,7 +1505,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
         <x:v>test</x:v>
@@ -1549,7 +1549,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
         <x:v>test</x:v>
@@ -1813,7 +1813,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
         <x:v>test</x:v>
@@ -1857,7 +1857,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
         <x:v>test</x:v>
@@ -1901,7 +1901,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
         <x:v>test</x:v>
@@ -1945,7 +1945,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
         <x:v>test</x:v>
@@ -1989,7 +1989,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
         <x:v>test</x:v>
@@ -2035,7 +2035,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R634f9144e3894cd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d3a9548a5343a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2044,9 +2044,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="8.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="8.890000343322754" hidden="0" customWidth="1"/>
@@ -2121,7 +2121,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>Completed comparable</x:v>
@@ -2185,7 +2185,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>Completed comparable</x:v>
@@ -2249,7 +2249,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
         <x:v>Completed comparable</x:v>
@@ -2283,7 +2283,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75ccf68335934f69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83413c1eb4d94efe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2292,11 +2292,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="57.779998779296875" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="7.78000020980835" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="13.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="16.110000610351562" hidden="0" customWidth="1"/>
@@ -2369,7 +2369,7 @@
         <x:v>TreeX</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Published</x:v>
+        <x:v>Unsupervised parameterised</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
         <x:v>treex_for_instance_exact_path_subset</x:v>
@@ -2410,10 +2410,14 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>aligned_predictions_and_evaluation_files</x:v>
-      </x:c>
-      <x:c r="F6" s="14"/>
-      <x:c r="G6" s="14"/>
+        <x:v>aligned_instance_and_semantic_predictions</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="n">
+        <x:v>6272039402</x:v>
+      </x:c>
       <x:c r="H6" s="12" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
@@ -2429,7 +2433,7 @@
         <x:v>SegmentAnyTree</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
         <x:v>segmentanytree_for-instance_fine_tuned_on_dev_20260711_002931</x:v>
@@ -2438,10 +2442,14 @@
         <x:v>test</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
-        <x:v>aligned_predictions_and_evaluation_files</x:v>
-      </x:c>
-      <x:c r="F7" s="14"/>
-      <x:c r="G7" s="14"/>
+        <x:v>aligned_instance_and_semantic_predictions</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="n">
+        <x:v>6270761232</x:v>
+      </x:c>
       <x:c r="H7" s="12" t="str">
         <x:v>retention_verified</x:v>
       </x:c>
@@ -2471,7 +2479,9 @@
       <x:c r="F8" s="14" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="G8" s="14"/>
+      <x:c r="G8" s="14" t="n">
+        <x:v>4694894674</x:v>
+      </x:c>
       <x:c r="H8" s="12" t="str">
         <x:v>sha256_verified</x:v>
       </x:c>
@@ -2487,7 +2497,7 @@
         <x:v>TreeLearn</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Fine-tuned</x:v>
+        <x:v>Fine-tuned on development data</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>treelearn_for-instance_fine_tuned_on_dev_long_20260712_233227</x:v>
@@ -2501,7 +2511,9 @@
       <x:c r="F9" s="14" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="G9" s="14"/>
+      <x:c r="G9" s="14" t="n">
+        <x:v>4547400887</x:v>
+      </x:c>
       <x:c r="H9" s="12" t="str">
         <x:v>sha256_verified</x:v>
       </x:c>
@@ -2519,7 +2531,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc29d11cfbd45465f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c4b8fa93a294c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>